<commit_message>
feat: add bottom borders and dynamic row insertion
</commit_message>
<xml_diff>
--- a/static/templates/tec02-A_template.xlsx
+++ b/static/templates/tec02-A_template.xlsx
@@ -176,7 +176,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="57">
+  <borders count="60">
     <border>
       <left/>
       <right/>
@@ -736,11 +736,35 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="47"/>
   </cellStyleXfs>
-  <cellXfs count="122">
+  <cellXfs count="125">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -1037,6 +1061,11 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="47" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="57" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="58" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="59" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1957,36 +1986,235 @@
     </row>
     <row r="24" ht="14.5" customHeight="1">
       <c r="A24" s="1" t="n"/>
-      <c r="B24" s="110" t="n"/>
-      <c r="AA24" s="111" t="n"/>
+      <c r="B24" s="122" t="n"/>
+      <c r="C24" s="123" t="n"/>
+      <c r="D24" s="123" t="n"/>
+      <c r="E24" s="123" t="n"/>
+      <c r="F24" s="123" t="n"/>
+      <c r="G24" s="123" t="n"/>
+      <c r="H24" s="123" t="n"/>
+      <c r="I24" s="123" t="n"/>
+      <c r="J24" s="123" t="n"/>
+      <c r="K24" s="123" t="n"/>
+      <c r="L24" s="123" t="n"/>
+      <c r="M24" s="123" t="n"/>
+      <c r="N24" s="123" t="n"/>
+      <c r="O24" s="123" t="n"/>
+      <c r="P24" s="123" t="n"/>
+      <c r="Q24" s="123" t="n"/>
+      <c r="R24" s="123" t="n"/>
+      <c r="S24" s="123" t="n"/>
+      <c r="T24" s="123" t="n"/>
+      <c r="U24" s="123" t="n"/>
+      <c r="V24" s="123" t="n"/>
+      <c r="W24" s="123" t="n"/>
+      <c r="X24" s="123" t="n"/>
+      <c r="Y24" s="123" t="n"/>
+      <c r="Z24" s="123" t="n"/>
+      <c r="AA24" s="124" t="n"/>
     </row>
     <row r="25" ht="14.5" customHeight="1">
       <c r="A25" s="1" t="n"/>
-      <c r="B25" s="110" t="n"/>
+      <c r="B25" s="122" t="n"/>
+      <c r="C25" s="123" t="n"/>
+      <c r="D25" s="123" t="n"/>
+      <c r="E25" s="123" t="n"/>
+      <c r="F25" s="123" t="n"/>
+      <c r="G25" s="123" t="n"/>
+      <c r="H25" s="123" t="n"/>
+      <c r="I25" s="123" t="n"/>
+      <c r="J25" s="123" t="n"/>
+      <c r="K25" s="123" t="n"/>
+      <c r="L25" s="123" t="n"/>
+      <c r="M25" s="123" t="n"/>
+      <c r="N25" s="123" t="n"/>
+      <c r="O25" s="123" t="n"/>
+      <c r="P25" s="123" t="n"/>
+      <c r="Q25" s="123" t="n"/>
+      <c r="R25" s="123" t="n"/>
+      <c r="S25" s="123" t="n"/>
+      <c r="T25" s="123" t="n"/>
+      <c r="U25" s="123" t="n"/>
+      <c r="V25" s="123" t="n"/>
+      <c r="W25" s="123" t="n"/>
+      <c r="X25" s="123" t="n"/>
+      <c r="Y25" s="123" t="n"/>
+      <c r="Z25" s="123" t="n"/>
+      <c r="AA25" s="124" t="n"/>
     </row>
     <row r="26" ht="14.5" customHeight="1">
       <c r="A26" s="1" t="n"/>
-      <c r="B26" s="110" t="n"/>
+      <c r="B26" s="122" t="n"/>
+      <c r="C26" s="123" t="n"/>
+      <c r="D26" s="123" t="n"/>
+      <c r="E26" s="123" t="n"/>
+      <c r="F26" s="123" t="n"/>
+      <c r="G26" s="123" t="n"/>
+      <c r="H26" s="123" t="n"/>
+      <c r="I26" s="123" t="n"/>
+      <c r="J26" s="123" t="n"/>
+      <c r="K26" s="123" t="n"/>
+      <c r="L26" s="123" t="n"/>
+      <c r="M26" s="123" t="n"/>
+      <c r="N26" s="123" t="n"/>
+      <c r="O26" s="123" t="n"/>
+      <c r="P26" s="123" t="n"/>
+      <c r="Q26" s="123" t="n"/>
+      <c r="R26" s="123" t="n"/>
+      <c r="S26" s="123" t="n"/>
+      <c r="T26" s="123" t="n"/>
+      <c r="U26" s="123" t="n"/>
+      <c r="V26" s="123" t="n"/>
+      <c r="W26" s="123" t="n"/>
+      <c r="X26" s="123" t="n"/>
+      <c r="Y26" s="123" t="n"/>
+      <c r="Z26" s="123" t="n"/>
+      <c r="AA26" s="124" t="n"/>
     </row>
     <row r="27" ht="14.5" customHeight="1">
       <c r="A27" s="1" t="n"/>
-      <c r="B27" s="110" t="n"/>
+      <c r="B27" s="122" t="n"/>
+      <c r="C27" s="123" t="n"/>
+      <c r="D27" s="123" t="n"/>
+      <c r="E27" s="123" t="n"/>
+      <c r="F27" s="123" t="n"/>
+      <c r="G27" s="123" t="n"/>
+      <c r="H27" s="123" t="n"/>
+      <c r="I27" s="123" t="n"/>
+      <c r="J27" s="123" t="n"/>
+      <c r="K27" s="123" t="n"/>
+      <c r="L27" s="123" t="n"/>
+      <c r="M27" s="123" t="n"/>
+      <c r="N27" s="123" t="n"/>
+      <c r="O27" s="123" t="n"/>
+      <c r="P27" s="123" t="n"/>
+      <c r="Q27" s="123" t="n"/>
+      <c r="R27" s="123" t="n"/>
+      <c r="S27" s="123" t="n"/>
+      <c r="T27" s="123" t="n"/>
+      <c r="U27" s="123" t="n"/>
+      <c r="V27" s="123" t="n"/>
+      <c r="W27" s="123" t="n"/>
+      <c r="X27" s="123" t="n"/>
+      <c r="Y27" s="123" t="n"/>
+      <c r="Z27" s="123" t="n"/>
+      <c r="AA27" s="124" t="n"/>
     </row>
     <row r="28" ht="14.5" customHeight="1">
       <c r="A28" s="1" t="n"/>
-      <c r="B28" s="110" t="n"/>
+      <c r="B28" s="122" t="n"/>
+      <c r="C28" s="123" t="n"/>
+      <c r="D28" s="123" t="n"/>
+      <c r="E28" s="123" t="n"/>
+      <c r="F28" s="123" t="n"/>
+      <c r="G28" s="123" t="n"/>
+      <c r="H28" s="123" t="n"/>
+      <c r="I28" s="123" t="n"/>
+      <c r="J28" s="123" t="n"/>
+      <c r="K28" s="123" t="n"/>
+      <c r="L28" s="123" t="n"/>
+      <c r="M28" s="123" t="n"/>
+      <c r="N28" s="123" t="n"/>
+      <c r="O28" s="123" t="n"/>
+      <c r="P28" s="123" t="n"/>
+      <c r="Q28" s="123" t="n"/>
+      <c r="R28" s="123" t="n"/>
+      <c r="S28" s="123" t="n"/>
+      <c r="T28" s="123" t="n"/>
+      <c r="U28" s="123" t="n"/>
+      <c r="V28" s="123" t="n"/>
+      <c r="W28" s="123" t="n"/>
+      <c r="X28" s="123" t="n"/>
+      <c r="Y28" s="123" t="n"/>
+      <c r="Z28" s="123" t="n"/>
+      <c r="AA28" s="124" t="n"/>
     </row>
     <row r="29" ht="14.5" customHeight="1">
       <c r="A29" s="1" t="n"/>
-      <c r="B29" s="110" t="n"/>
+      <c r="B29" s="122" t="n"/>
+      <c r="C29" s="123" t="n"/>
+      <c r="D29" s="123" t="n"/>
+      <c r="E29" s="123" t="n"/>
+      <c r="F29" s="123" t="n"/>
+      <c r="G29" s="123" t="n"/>
+      <c r="H29" s="123" t="n"/>
+      <c r="I29" s="123" t="n"/>
+      <c r="J29" s="123" t="n"/>
+      <c r="K29" s="123" t="n"/>
+      <c r="L29" s="123" t="n"/>
+      <c r="M29" s="123" t="n"/>
+      <c r="N29" s="123" t="n"/>
+      <c r="O29" s="123" t="n"/>
+      <c r="P29" s="123" t="n"/>
+      <c r="Q29" s="123" t="n"/>
+      <c r="R29" s="123" t="n"/>
+      <c r="S29" s="123" t="n"/>
+      <c r="T29" s="123" t="n"/>
+      <c r="U29" s="123" t="n"/>
+      <c r="V29" s="123" t="n"/>
+      <c r="W29" s="123" t="n"/>
+      <c r="X29" s="123" t="n"/>
+      <c r="Y29" s="123" t="n"/>
+      <c r="Z29" s="123" t="n"/>
+      <c r="AA29" s="124" t="n"/>
     </row>
     <row r="30" ht="14.5" customHeight="1">
       <c r="A30" s="1" t="n"/>
-      <c r="B30" s="110" t="n"/>
+      <c r="B30" s="122" t="n"/>
+      <c r="C30" s="123" t="n"/>
+      <c r="D30" s="123" t="n"/>
+      <c r="E30" s="123" t="n"/>
+      <c r="F30" s="123" t="n"/>
+      <c r="G30" s="123" t="n"/>
+      <c r="H30" s="123" t="n"/>
+      <c r="I30" s="123" t="n"/>
+      <c r="J30" s="123" t="n"/>
+      <c r="K30" s="123" t="n"/>
+      <c r="L30" s="123" t="n"/>
+      <c r="M30" s="123" t="n"/>
+      <c r="N30" s="123" t="n"/>
+      <c r="O30" s="123" t="n"/>
+      <c r="P30" s="123" t="n"/>
+      <c r="Q30" s="123" t="n"/>
+      <c r="R30" s="123" t="n"/>
+      <c r="S30" s="123" t="n"/>
+      <c r="T30" s="123" t="n"/>
+      <c r="U30" s="123" t="n"/>
+      <c r="V30" s="123" t="n"/>
+      <c r="W30" s="123" t="n"/>
+      <c r="X30" s="123" t="n"/>
+      <c r="Y30" s="123" t="n"/>
+      <c r="Z30" s="123" t="n"/>
+      <c r="AA30" s="124" t="n"/>
     </row>
     <row r="31" ht="14.5" customHeight="1">
       <c r="A31" s="1" t="n"/>
-      <c r="B31" s="110" t="n"/>
+      <c r="B31" s="122" t="n"/>
+      <c r="C31" s="123" t="n"/>
+      <c r="D31" s="123" t="n"/>
+      <c r="E31" s="123" t="n"/>
+      <c r="F31" s="123" t="n"/>
+      <c r="G31" s="123" t="n"/>
+      <c r="H31" s="123" t="n"/>
+      <c r="I31" s="123" t="n"/>
+      <c r="J31" s="123" t="n"/>
+      <c r="K31" s="123" t="n"/>
+      <c r="L31" s="123" t="n"/>
+      <c r="M31" s="123" t="n"/>
+      <c r="N31" s="123" t="n"/>
+      <c r="O31" s="123" t="n"/>
+      <c r="P31" s="123" t="n"/>
+      <c r="Q31" s="123" t="n"/>
+      <c r="R31" s="123" t="n"/>
+      <c r="S31" s="123" t="n"/>
+      <c r="T31" s="123" t="n"/>
+      <c r="U31" s="123" t="n"/>
+      <c r="V31" s="123" t="n"/>
+      <c r="W31" s="123" t="n"/>
+      <c r="X31" s="123" t="n"/>
+      <c r="Y31" s="123" t="n"/>
+      <c r="Z31" s="123" t="n"/>
+      <c r="AA31" s="124" t="n"/>
     </row>
     <row r="32" ht="15" customHeight="1">
       <c r="A32" s="1" t="n"/>
@@ -2023,32 +2251,206 @@
     </row>
     <row r="33" ht="14.5" customHeight="1">
       <c r="A33" s="1" t="n"/>
-      <c r="B33" s="110" t="n"/>
-      <c r="AA33" s="111" t="n"/>
+      <c r="B33" s="122" t="n"/>
+      <c r="C33" s="123" t="n"/>
+      <c r="D33" s="123" t="n"/>
+      <c r="E33" s="123" t="n"/>
+      <c r="F33" s="123" t="n"/>
+      <c r="G33" s="123" t="n"/>
+      <c r="H33" s="123" t="n"/>
+      <c r="I33" s="123" t="n"/>
+      <c r="J33" s="123" t="n"/>
+      <c r="K33" s="123" t="n"/>
+      <c r="L33" s="123" t="n"/>
+      <c r="M33" s="123" t="n"/>
+      <c r="N33" s="123" t="n"/>
+      <c r="O33" s="123" t="n"/>
+      <c r="P33" s="123" t="n"/>
+      <c r="Q33" s="123" t="n"/>
+      <c r="R33" s="123" t="n"/>
+      <c r="S33" s="123" t="n"/>
+      <c r="T33" s="123" t="n"/>
+      <c r="U33" s="123" t="n"/>
+      <c r="V33" s="123" t="n"/>
+      <c r="W33" s="123" t="n"/>
+      <c r="X33" s="123" t="n"/>
+      <c r="Y33" s="123" t="n"/>
+      <c r="Z33" s="123" t="n"/>
+      <c r="AA33" s="124" t="n"/>
     </row>
     <row r="34" ht="14.5" customHeight="1">
       <c r="A34" s="1" t="n"/>
-      <c r="B34" s="110" t="n"/>
+      <c r="B34" s="122" t="n"/>
+      <c r="C34" s="123" t="n"/>
+      <c r="D34" s="123" t="n"/>
+      <c r="E34" s="123" t="n"/>
+      <c r="F34" s="123" t="n"/>
+      <c r="G34" s="123" t="n"/>
+      <c r="H34" s="123" t="n"/>
+      <c r="I34" s="123" t="n"/>
+      <c r="J34" s="123" t="n"/>
+      <c r="K34" s="123" t="n"/>
+      <c r="L34" s="123" t="n"/>
+      <c r="M34" s="123" t="n"/>
+      <c r="N34" s="123" t="n"/>
+      <c r="O34" s="123" t="n"/>
+      <c r="P34" s="123" t="n"/>
+      <c r="Q34" s="123" t="n"/>
+      <c r="R34" s="123" t="n"/>
+      <c r="S34" s="123" t="n"/>
+      <c r="T34" s="123" t="n"/>
+      <c r="U34" s="123" t="n"/>
+      <c r="V34" s="123" t="n"/>
+      <c r="W34" s="123" t="n"/>
+      <c r="X34" s="123" t="n"/>
+      <c r="Y34" s="123" t="n"/>
+      <c r="Z34" s="123" t="n"/>
+      <c r="AA34" s="124" t="n"/>
     </row>
     <row r="35" ht="14.5" customHeight="1">
       <c r="A35" s="1" t="n"/>
-      <c r="B35" s="110" t="n"/>
+      <c r="B35" s="122" t="n"/>
+      <c r="C35" s="123" t="n"/>
+      <c r="D35" s="123" t="n"/>
+      <c r="E35" s="123" t="n"/>
+      <c r="F35" s="123" t="n"/>
+      <c r="G35" s="123" t="n"/>
+      <c r="H35" s="123" t="n"/>
+      <c r="I35" s="123" t="n"/>
+      <c r="J35" s="123" t="n"/>
+      <c r="K35" s="123" t="n"/>
+      <c r="L35" s="123" t="n"/>
+      <c r="M35" s="123" t="n"/>
+      <c r="N35" s="123" t="n"/>
+      <c r="O35" s="123" t="n"/>
+      <c r="P35" s="123" t="n"/>
+      <c r="Q35" s="123" t="n"/>
+      <c r="R35" s="123" t="n"/>
+      <c r="S35" s="123" t="n"/>
+      <c r="T35" s="123" t="n"/>
+      <c r="U35" s="123" t="n"/>
+      <c r="V35" s="123" t="n"/>
+      <c r="W35" s="123" t="n"/>
+      <c r="X35" s="123" t="n"/>
+      <c r="Y35" s="123" t="n"/>
+      <c r="Z35" s="123" t="n"/>
+      <c r="AA35" s="124" t="n"/>
     </row>
     <row r="36" ht="14.5" customHeight="1">
       <c r="A36" s="1" t="n"/>
-      <c r="B36" s="110" t="n"/>
+      <c r="B36" s="122" t="n"/>
+      <c r="C36" s="123" t="n"/>
+      <c r="D36" s="123" t="n"/>
+      <c r="E36" s="123" t="n"/>
+      <c r="F36" s="123" t="n"/>
+      <c r="G36" s="123" t="n"/>
+      <c r="H36" s="123" t="n"/>
+      <c r="I36" s="123" t="n"/>
+      <c r="J36" s="123" t="n"/>
+      <c r="K36" s="123" t="n"/>
+      <c r="L36" s="123" t="n"/>
+      <c r="M36" s="123" t="n"/>
+      <c r="N36" s="123" t="n"/>
+      <c r="O36" s="123" t="n"/>
+      <c r="P36" s="123" t="n"/>
+      <c r="Q36" s="123" t="n"/>
+      <c r="R36" s="123" t="n"/>
+      <c r="S36" s="123" t="n"/>
+      <c r="T36" s="123" t="n"/>
+      <c r="U36" s="123" t="n"/>
+      <c r="V36" s="123" t="n"/>
+      <c r="W36" s="123" t="n"/>
+      <c r="X36" s="123" t="n"/>
+      <c r="Y36" s="123" t="n"/>
+      <c r="Z36" s="123" t="n"/>
+      <c r="AA36" s="124" t="n"/>
     </row>
     <row r="37" ht="14.5" customHeight="1">
       <c r="A37" s="1" t="n"/>
-      <c r="B37" s="110" t="n"/>
+      <c r="B37" s="122" t="n"/>
+      <c r="C37" s="123" t="n"/>
+      <c r="D37" s="123" t="n"/>
+      <c r="E37" s="123" t="n"/>
+      <c r="F37" s="123" t="n"/>
+      <c r="G37" s="123" t="n"/>
+      <c r="H37" s="123" t="n"/>
+      <c r="I37" s="123" t="n"/>
+      <c r="J37" s="123" t="n"/>
+      <c r="K37" s="123" t="n"/>
+      <c r="L37" s="123" t="n"/>
+      <c r="M37" s="123" t="n"/>
+      <c r="N37" s="123" t="n"/>
+      <c r="O37" s="123" t="n"/>
+      <c r="P37" s="123" t="n"/>
+      <c r="Q37" s="123" t="n"/>
+      <c r="R37" s="123" t="n"/>
+      <c r="S37" s="123" t="n"/>
+      <c r="T37" s="123" t="n"/>
+      <c r="U37" s="123" t="n"/>
+      <c r="V37" s="123" t="n"/>
+      <c r="W37" s="123" t="n"/>
+      <c r="X37" s="123" t="n"/>
+      <c r="Y37" s="123" t="n"/>
+      <c r="Z37" s="123" t="n"/>
+      <c r="AA37" s="124" t="n"/>
     </row>
     <row r="38" ht="14.5" customHeight="1">
       <c r="A38" s="1" t="n"/>
-      <c r="B38" s="110" t="n"/>
+      <c r="B38" s="122" t="n"/>
+      <c r="C38" s="123" t="n"/>
+      <c r="D38" s="123" t="n"/>
+      <c r="E38" s="123" t="n"/>
+      <c r="F38" s="123" t="n"/>
+      <c r="G38" s="123" t="n"/>
+      <c r="H38" s="123" t="n"/>
+      <c r="I38" s="123" t="n"/>
+      <c r="J38" s="123" t="n"/>
+      <c r="K38" s="123" t="n"/>
+      <c r="L38" s="123" t="n"/>
+      <c r="M38" s="123" t="n"/>
+      <c r="N38" s="123" t="n"/>
+      <c r="O38" s="123" t="n"/>
+      <c r="P38" s="123" t="n"/>
+      <c r="Q38" s="123" t="n"/>
+      <c r="R38" s="123" t="n"/>
+      <c r="S38" s="123" t="n"/>
+      <c r="T38" s="123" t="n"/>
+      <c r="U38" s="123" t="n"/>
+      <c r="V38" s="123" t="n"/>
+      <c r="W38" s="123" t="n"/>
+      <c r="X38" s="123" t="n"/>
+      <c r="Y38" s="123" t="n"/>
+      <c r="Z38" s="123" t="n"/>
+      <c r="AA38" s="124" t="n"/>
     </row>
     <row r="39" ht="14.5" customHeight="1">
       <c r="A39" s="1" t="n"/>
-      <c r="B39" s="110" t="n"/>
+      <c r="B39" s="122" t="n"/>
+      <c r="C39" s="123" t="n"/>
+      <c r="D39" s="123" t="n"/>
+      <c r="E39" s="123" t="n"/>
+      <c r="F39" s="123" t="n"/>
+      <c r="G39" s="123" t="n"/>
+      <c r="H39" s="123" t="n"/>
+      <c r="I39" s="123" t="n"/>
+      <c r="J39" s="123" t="n"/>
+      <c r="K39" s="123" t="n"/>
+      <c r="L39" s="123" t="n"/>
+      <c r="M39" s="123" t="n"/>
+      <c r="N39" s="123" t="n"/>
+      <c r="O39" s="123" t="n"/>
+      <c r="P39" s="123" t="n"/>
+      <c r="Q39" s="123" t="n"/>
+      <c r="R39" s="123" t="n"/>
+      <c r="S39" s="123" t="n"/>
+      <c r="T39" s="123" t="n"/>
+      <c r="U39" s="123" t="n"/>
+      <c r="V39" s="123" t="n"/>
+      <c r="W39" s="123" t="n"/>
+      <c r="X39" s="123" t="n"/>
+      <c r="Y39" s="123" t="n"/>
+      <c r="Z39" s="123" t="n"/>
+      <c r="AA39" s="124" t="n"/>
     </row>
     <row r="40" ht="15" customHeight="1">
       <c r="A40" s="1" t="n"/>
@@ -2085,56 +2487,206 @@
     </row>
     <row r="41" ht="14.5" customHeight="1">
       <c r="A41" s="1" t="n"/>
-      <c r="B41" s="115" t="n"/>
-      <c r="C41" s="116" t="n"/>
-      <c r="D41" s="116" t="n"/>
-      <c r="E41" s="116" t="n"/>
-      <c r="F41" s="116" t="n"/>
-      <c r="G41" s="116" t="n"/>
-      <c r="H41" s="116" t="n"/>
-      <c r="I41" s="116" t="n"/>
-      <c r="J41" s="116" t="n"/>
-      <c r="K41" s="116" t="n"/>
-      <c r="L41" s="116" t="n"/>
-      <c r="M41" s="116" t="n"/>
-      <c r="N41" s="116" t="n"/>
-      <c r="O41" s="116" t="n"/>
-      <c r="P41" s="116" t="n"/>
-      <c r="Q41" s="116" t="n"/>
-      <c r="R41" s="116" t="n"/>
-      <c r="S41" s="116" t="n"/>
-      <c r="T41" s="116" t="n"/>
-      <c r="U41" s="116" t="n"/>
-      <c r="V41" s="116" t="n"/>
-      <c r="W41" s="116" t="n"/>
-      <c r="X41" s="116" t="n"/>
-      <c r="Y41" s="116" t="n"/>
-      <c r="Z41" s="116" t="n"/>
-      <c r="AA41" s="117" t="n"/>
+      <c r="B41" s="122" t="n"/>
+      <c r="C41" s="123" t="n"/>
+      <c r="D41" s="123" t="n"/>
+      <c r="E41" s="123" t="n"/>
+      <c r="F41" s="123" t="n"/>
+      <c r="G41" s="123" t="n"/>
+      <c r="H41" s="123" t="n"/>
+      <c r="I41" s="123" t="n"/>
+      <c r="J41" s="123" t="n"/>
+      <c r="K41" s="123" t="n"/>
+      <c r="L41" s="123" t="n"/>
+      <c r="M41" s="123" t="n"/>
+      <c r="N41" s="123" t="n"/>
+      <c r="O41" s="123" t="n"/>
+      <c r="P41" s="123" t="n"/>
+      <c r="Q41" s="123" t="n"/>
+      <c r="R41" s="123" t="n"/>
+      <c r="S41" s="123" t="n"/>
+      <c r="T41" s="123" t="n"/>
+      <c r="U41" s="123" t="n"/>
+      <c r="V41" s="123" t="n"/>
+      <c r="W41" s="123" t="n"/>
+      <c r="X41" s="123" t="n"/>
+      <c r="Y41" s="123" t="n"/>
+      <c r="Z41" s="123" t="n"/>
+      <c r="AA41" s="124" t="n"/>
     </row>
     <row r="42" ht="14.5" customHeight="1">
       <c r="A42" s="1" t="n"/>
-      <c r="B42" s="115" t="n"/>
+      <c r="B42" s="122" t="n"/>
+      <c r="C42" s="123" t="n"/>
+      <c r="D42" s="123" t="n"/>
+      <c r="E42" s="123" t="n"/>
+      <c r="F42" s="123" t="n"/>
+      <c r="G42" s="123" t="n"/>
+      <c r="H42" s="123" t="n"/>
+      <c r="I42" s="123" t="n"/>
+      <c r="J42" s="123" t="n"/>
+      <c r="K42" s="123" t="n"/>
+      <c r="L42" s="123" t="n"/>
+      <c r="M42" s="123" t="n"/>
+      <c r="N42" s="123" t="n"/>
+      <c r="O42" s="123" t="n"/>
+      <c r="P42" s="123" t="n"/>
+      <c r="Q42" s="123" t="n"/>
+      <c r="R42" s="123" t="n"/>
+      <c r="S42" s="123" t="n"/>
+      <c r="T42" s="123" t="n"/>
+      <c r="U42" s="123" t="n"/>
+      <c r="V42" s="123" t="n"/>
+      <c r="W42" s="123" t="n"/>
+      <c r="X42" s="123" t="n"/>
+      <c r="Y42" s="123" t="n"/>
+      <c r="Z42" s="123" t="n"/>
+      <c r="AA42" s="124" t="n"/>
     </row>
     <row r="43" ht="14.5" customHeight="1">
       <c r="A43" s="1" t="n"/>
-      <c r="B43" s="115" t="n"/>
+      <c r="B43" s="122" t="n"/>
+      <c r="C43" s="123" t="n"/>
+      <c r="D43" s="123" t="n"/>
+      <c r="E43" s="123" t="n"/>
+      <c r="F43" s="123" t="n"/>
+      <c r="G43" s="123" t="n"/>
+      <c r="H43" s="123" t="n"/>
+      <c r="I43" s="123" t="n"/>
+      <c r="J43" s="123" t="n"/>
+      <c r="K43" s="123" t="n"/>
+      <c r="L43" s="123" t="n"/>
+      <c r="M43" s="123" t="n"/>
+      <c r="N43" s="123" t="n"/>
+      <c r="O43" s="123" t="n"/>
+      <c r="P43" s="123" t="n"/>
+      <c r="Q43" s="123" t="n"/>
+      <c r="R43" s="123" t="n"/>
+      <c r="S43" s="123" t="n"/>
+      <c r="T43" s="123" t="n"/>
+      <c r="U43" s="123" t="n"/>
+      <c r="V43" s="123" t="n"/>
+      <c r="W43" s="123" t="n"/>
+      <c r="X43" s="123" t="n"/>
+      <c r="Y43" s="123" t="n"/>
+      <c r="Z43" s="123" t="n"/>
+      <c r="AA43" s="124" t="n"/>
     </row>
     <row r="44" ht="14.5" customHeight="1">
       <c r="A44" s="1" t="n"/>
-      <c r="B44" s="115" t="n"/>
+      <c r="B44" s="122" t="n"/>
+      <c r="C44" s="123" t="n"/>
+      <c r="D44" s="123" t="n"/>
+      <c r="E44" s="123" t="n"/>
+      <c r="F44" s="123" t="n"/>
+      <c r="G44" s="123" t="n"/>
+      <c r="H44" s="123" t="n"/>
+      <c r="I44" s="123" t="n"/>
+      <c r="J44" s="123" t="n"/>
+      <c r="K44" s="123" t="n"/>
+      <c r="L44" s="123" t="n"/>
+      <c r="M44" s="123" t="n"/>
+      <c r="N44" s="123" t="n"/>
+      <c r="O44" s="123" t="n"/>
+      <c r="P44" s="123" t="n"/>
+      <c r="Q44" s="123" t="n"/>
+      <c r="R44" s="123" t="n"/>
+      <c r="S44" s="123" t="n"/>
+      <c r="T44" s="123" t="n"/>
+      <c r="U44" s="123" t="n"/>
+      <c r="V44" s="123" t="n"/>
+      <c r="W44" s="123" t="n"/>
+      <c r="X44" s="123" t="n"/>
+      <c r="Y44" s="123" t="n"/>
+      <c r="Z44" s="123" t="n"/>
+      <c r="AA44" s="124" t="n"/>
     </row>
     <row r="45" ht="14.5" customHeight="1">
       <c r="A45" s="1" t="n"/>
-      <c r="B45" s="115" t="n"/>
+      <c r="B45" s="122" t="n"/>
+      <c r="C45" s="123" t="n"/>
+      <c r="D45" s="123" t="n"/>
+      <c r="E45" s="123" t="n"/>
+      <c r="F45" s="123" t="n"/>
+      <c r="G45" s="123" t="n"/>
+      <c r="H45" s="123" t="n"/>
+      <c r="I45" s="123" t="n"/>
+      <c r="J45" s="123" t="n"/>
+      <c r="K45" s="123" t="n"/>
+      <c r="L45" s="123" t="n"/>
+      <c r="M45" s="123" t="n"/>
+      <c r="N45" s="123" t="n"/>
+      <c r="O45" s="123" t="n"/>
+      <c r="P45" s="123" t="n"/>
+      <c r="Q45" s="123" t="n"/>
+      <c r="R45" s="123" t="n"/>
+      <c r="S45" s="123" t="n"/>
+      <c r="T45" s="123" t="n"/>
+      <c r="U45" s="123" t="n"/>
+      <c r="V45" s="123" t="n"/>
+      <c r="W45" s="123" t="n"/>
+      <c r="X45" s="123" t="n"/>
+      <c r="Y45" s="123" t="n"/>
+      <c r="Z45" s="123" t="n"/>
+      <c r="AA45" s="124" t="n"/>
     </row>
     <row r="46" ht="14.5" customHeight="1">
       <c r="A46" s="1" t="n"/>
-      <c r="B46" s="115" t="n"/>
+      <c r="B46" s="122" t="n"/>
+      <c r="C46" s="123" t="n"/>
+      <c r="D46" s="123" t="n"/>
+      <c r="E46" s="123" t="n"/>
+      <c r="F46" s="123" t="n"/>
+      <c r="G46" s="123" t="n"/>
+      <c r="H46" s="123" t="n"/>
+      <c r="I46" s="123" t="n"/>
+      <c r="J46" s="123" t="n"/>
+      <c r="K46" s="123" t="n"/>
+      <c r="L46" s="123" t="n"/>
+      <c r="M46" s="123" t="n"/>
+      <c r="N46" s="123" t="n"/>
+      <c r="O46" s="123" t="n"/>
+      <c r="P46" s="123" t="n"/>
+      <c r="Q46" s="123" t="n"/>
+      <c r="R46" s="123" t="n"/>
+      <c r="S46" s="123" t="n"/>
+      <c r="T46" s="123" t="n"/>
+      <c r="U46" s="123" t="n"/>
+      <c r="V46" s="123" t="n"/>
+      <c r="W46" s="123" t="n"/>
+      <c r="X46" s="123" t="n"/>
+      <c r="Y46" s="123" t="n"/>
+      <c r="Z46" s="123" t="n"/>
+      <c r="AA46" s="124" t="n"/>
     </row>
     <row r="47" ht="14.5" customHeight="1">
       <c r="A47" s="1" t="n"/>
-      <c r="B47" s="115" t="n"/>
+      <c r="B47" s="122" t="n"/>
+      <c r="C47" s="123" t="n"/>
+      <c r="D47" s="123" t="n"/>
+      <c r="E47" s="123" t="n"/>
+      <c r="F47" s="123" t="n"/>
+      <c r="G47" s="123" t="n"/>
+      <c r="H47" s="123" t="n"/>
+      <c r="I47" s="123" t="n"/>
+      <c r="J47" s="123" t="n"/>
+      <c r="K47" s="123" t="n"/>
+      <c r="L47" s="123" t="n"/>
+      <c r="M47" s="123" t="n"/>
+      <c r="N47" s="123" t="n"/>
+      <c r="O47" s="123" t="n"/>
+      <c r="P47" s="123" t="n"/>
+      <c r="Q47" s="123" t="n"/>
+      <c r="R47" s="123" t="n"/>
+      <c r="S47" s="123" t="n"/>
+      <c r="T47" s="123" t="n"/>
+      <c r="U47" s="123" t="n"/>
+      <c r="V47" s="123" t="n"/>
+      <c r="W47" s="123" t="n"/>
+      <c r="X47" s="123" t="n"/>
+      <c r="Y47" s="123" t="n"/>
+      <c r="Z47" s="123" t="n"/>
+      <c r="AA47" s="124" t="n"/>
     </row>
     <row r="48" ht="15" customHeight="1">
       <c r="A48" s="1" t="n"/>
@@ -2171,56 +2723,206 @@
     </row>
     <row r="49" ht="14.5" customHeight="1">
       <c r="A49" s="30" t="n"/>
-      <c r="B49" s="119" t="n"/>
-      <c r="C49" s="105" t="n"/>
-      <c r="D49" s="105" t="n"/>
-      <c r="E49" s="105" t="n"/>
-      <c r="F49" s="105" t="n"/>
-      <c r="G49" s="105" t="n"/>
-      <c r="H49" s="105" t="n"/>
-      <c r="I49" s="105" t="n"/>
-      <c r="J49" s="105" t="n"/>
-      <c r="K49" s="105" t="n"/>
-      <c r="L49" s="105" t="n"/>
-      <c r="M49" s="105" t="n"/>
-      <c r="N49" s="105" t="n"/>
-      <c r="O49" s="105" t="n"/>
-      <c r="P49" s="105" t="n"/>
-      <c r="Q49" s="105" t="n"/>
-      <c r="R49" s="105" t="n"/>
-      <c r="S49" s="105" t="n"/>
-      <c r="T49" s="105" t="n"/>
-      <c r="U49" s="105" t="n"/>
-      <c r="V49" s="105" t="n"/>
-      <c r="W49" s="105" t="n"/>
-      <c r="X49" s="105" t="n"/>
-      <c r="Y49" s="105" t="n"/>
-      <c r="Z49" s="105" t="n"/>
-      <c r="AA49" s="106" t="n"/>
+      <c r="B49" s="122" t="n"/>
+      <c r="C49" s="123" t="n"/>
+      <c r="D49" s="123" t="n"/>
+      <c r="E49" s="123" t="n"/>
+      <c r="F49" s="123" t="n"/>
+      <c r="G49" s="123" t="n"/>
+      <c r="H49" s="123" t="n"/>
+      <c r="I49" s="123" t="n"/>
+      <c r="J49" s="123" t="n"/>
+      <c r="K49" s="123" t="n"/>
+      <c r="L49" s="123" t="n"/>
+      <c r="M49" s="123" t="n"/>
+      <c r="N49" s="123" t="n"/>
+      <c r="O49" s="123" t="n"/>
+      <c r="P49" s="123" t="n"/>
+      <c r="Q49" s="123" t="n"/>
+      <c r="R49" s="123" t="n"/>
+      <c r="S49" s="123" t="n"/>
+      <c r="T49" s="123" t="n"/>
+      <c r="U49" s="123" t="n"/>
+      <c r="V49" s="123" t="n"/>
+      <c r="W49" s="123" t="n"/>
+      <c r="X49" s="123" t="n"/>
+      <c r="Y49" s="123" t="n"/>
+      <c r="Z49" s="123" t="n"/>
+      <c r="AA49" s="124" t="n"/>
     </row>
     <row r="50" ht="14.5" customHeight="1">
       <c r="A50" s="30" t="n"/>
-      <c r="B50" s="119" t="n"/>
+      <c r="B50" s="122" t="n"/>
+      <c r="C50" s="123" t="n"/>
+      <c r="D50" s="123" t="n"/>
+      <c r="E50" s="123" t="n"/>
+      <c r="F50" s="123" t="n"/>
+      <c r="G50" s="123" t="n"/>
+      <c r="H50" s="123" t="n"/>
+      <c r="I50" s="123" t="n"/>
+      <c r="J50" s="123" t="n"/>
+      <c r="K50" s="123" t="n"/>
+      <c r="L50" s="123" t="n"/>
+      <c r="M50" s="123" t="n"/>
+      <c r="N50" s="123" t="n"/>
+      <c r="O50" s="123" t="n"/>
+      <c r="P50" s="123" t="n"/>
+      <c r="Q50" s="123" t="n"/>
+      <c r="R50" s="123" t="n"/>
+      <c r="S50" s="123" t="n"/>
+      <c r="T50" s="123" t="n"/>
+      <c r="U50" s="123" t="n"/>
+      <c r="V50" s="123" t="n"/>
+      <c r="W50" s="123" t="n"/>
+      <c r="X50" s="123" t="n"/>
+      <c r="Y50" s="123" t="n"/>
+      <c r="Z50" s="123" t="n"/>
+      <c r="AA50" s="124" t="n"/>
     </row>
     <row r="51" ht="14.5" customHeight="1">
       <c r="A51" s="30" t="n"/>
-      <c r="B51" s="119" t="n"/>
+      <c r="B51" s="122" t="n"/>
+      <c r="C51" s="123" t="n"/>
+      <c r="D51" s="123" t="n"/>
+      <c r="E51" s="123" t="n"/>
+      <c r="F51" s="123" t="n"/>
+      <c r="G51" s="123" t="n"/>
+      <c r="H51" s="123" t="n"/>
+      <c r="I51" s="123" t="n"/>
+      <c r="J51" s="123" t="n"/>
+      <c r="K51" s="123" t="n"/>
+      <c r="L51" s="123" t="n"/>
+      <c r="M51" s="123" t="n"/>
+      <c r="N51" s="123" t="n"/>
+      <c r="O51" s="123" t="n"/>
+      <c r="P51" s="123" t="n"/>
+      <c r="Q51" s="123" t="n"/>
+      <c r="R51" s="123" t="n"/>
+      <c r="S51" s="123" t="n"/>
+      <c r="T51" s="123" t="n"/>
+      <c r="U51" s="123" t="n"/>
+      <c r="V51" s="123" t="n"/>
+      <c r="W51" s="123" t="n"/>
+      <c r="X51" s="123" t="n"/>
+      <c r="Y51" s="123" t="n"/>
+      <c r="Z51" s="123" t="n"/>
+      <c r="AA51" s="124" t="n"/>
     </row>
     <row r="52" ht="14.5" customHeight="1">
       <c r="A52" s="30" t="n"/>
-      <c r="B52" s="119" t="n"/>
+      <c r="B52" s="122" t="n"/>
+      <c r="C52" s="123" t="n"/>
+      <c r="D52" s="123" t="n"/>
+      <c r="E52" s="123" t="n"/>
+      <c r="F52" s="123" t="n"/>
+      <c r="G52" s="123" t="n"/>
+      <c r="H52" s="123" t="n"/>
+      <c r="I52" s="123" t="n"/>
+      <c r="J52" s="123" t="n"/>
+      <c r="K52" s="123" t="n"/>
+      <c r="L52" s="123" t="n"/>
+      <c r="M52" s="123" t="n"/>
+      <c r="N52" s="123" t="n"/>
+      <c r="O52" s="123" t="n"/>
+      <c r="P52" s="123" t="n"/>
+      <c r="Q52" s="123" t="n"/>
+      <c r="R52" s="123" t="n"/>
+      <c r="S52" s="123" t="n"/>
+      <c r="T52" s="123" t="n"/>
+      <c r="U52" s="123" t="n"/>
+      <c r="V52" s="123" t="n"/>
+      <c r="W52" s="123" t="n"/>
+      <c r="X52" s="123" t="n"/>
+      <c r="Y52" s="123" t="n"/>
+      <c r="Z52" s="123" t="n"/>
+      <c r="AA52" s="124" t="n"/>
     </row>
     <row r="53" ht="14.5" customHeight="1">
       <c r="A53" s="30" t="n"/>
-      <c r="B53" s="119" t="n"/>
+      <c r="B53" s="122" t="n"/>
+      <c r="C53" s="123" t="n"/>
+      <c r="D53" s="123" t="n"/>
+      <c r="E53" s="123" t="n"/>
+      <c r="F53" s="123" t="n"/>
+      <c r="G53" s="123" t="n"/>
+      <c r="H53" s="123" t="n"/>
+      <c r="I53" s="123" t="n"/>
+      <c r="J53" s="123" t="n"/>
+      <c r="K53" s="123" t="n"/>
+      <c r="L53" s="123" t="n"/>
+      <c r="M53" s="123" t="n"/>
+      <c r="N53" s="123" t="n"/>
+      <c r="O53" s="123" t="n"/>
+      <c r="P53" s="123" t="n"/>
+      <c r="Q53" s="123" t="n"/>
+      <c r="R53" s="123" t="n"/>
+      <c r="S53" s="123" t="n"/>
+      <c r="T53" s="123" t="n"/>
+      <c r="U53" s="123" t="n"/>
+      <c r="V53" s="123" t="n"/>
+      <c r="W53" s="123" t="n"/>
+      <c r="X53" s="123" t="n"/>
+      <c r="Y53" s="123" t="n"/>
+      <c r="Z53" s="123" t="n"/>
+      <c r="AA53" s="124" t="n"/>
     </row>
     <row r="54" ht="14.5" customHeight="1">
       <c r="A54" s="30" t="n"/>
-      <c r="B54" s="119" t="n"/>
+      <c r="B54" s="122" t="n"/>
+      <c r="C54" s="123" t="n"/>
+      <c r="D54" s="123" t="n"/>
+      <c r="E54" s="123" t="n"/>
+      <c r="F54" s="123" t="n"/>
+      <c r="G54" s="123" t="n"/>
+      <c r="H54" s="123" t="n"/>
+      <c r="I54" s="123" t="n"/>
+      <c r="J54" s="123" t="n"/>
+      <c r="K54" s="123" t="n"/>
+      <c r="L54" s="123" t="n"/>
+      <c r="M54" s="123" t="n"/>
+      <c r="N54" s="123" t="n"/>
+      <c r="O54" s="123" t="n"/>
+      <c r="P54" s="123" t="n"/>
+      <c r="Q54" s="123" t="n"/>
+      <c r="R54" s="123" t="n"/>
+      <c r="S54" s="123" t="n"/>
+      <c r="T54" s="123" t="n"/>
+      <c r="U54" s="123" t="n"/>
+      <c r="V54" s="123" t="n"/>
+      <c r="W54" s="123" t="n"/>
+      <c r="X54" s="123" t="n"/>
+      <c r="Y54" s="123" t="n"/>
+      <c r="Z54" s="123" t="n"/>
+      <c r="AA54" s="124" t="n"/>
     </row>
     <row r="55" ht="14.5" customHeight="1">
       <c r="A55" s="30" t="n"/>
-      <c r="B55" s="119" t="n"/>
+      <c r="B55" s="122" t="n"/>
+      <c r="C55" s="123" t="n"/>
+      <c r="D55" s="123" t="n"/>
+      <c r="E55" s="123" t="n"/>
+      <c r="F55" s="123" t="n"/>
+      <c r="G55" s="123" t="n"/>
+      <c r="H55" s="123" t="n"/>
+      <c r="I55" s="123" t="n"/>
+      <c r="J55" s="123" t="n"/>
+      <c r="K55" s="123" t="n"/>
+      <c r="L55" s="123" t="n"/>
+      <c r="M55" s="123" t="n"/>
+      <c r="N55" s="123" t="n"/>
+      <c r="O55" s="123" t="n"/>
+      <c r="P55" s="123" t="n"/>
+      <c r="Q55" s="123" t="n"/>
+      <c r="R55" s="123" t="n"/>
+      <c r="S55" s="123" t="n"/>
+      <c r="T55" s="123" t="n"/>
+      <c r="U55" s="123" t="n"/>
+      <c r="V55" s="123" t="n"/>
+      <c r="W55" s="123" t="n"/>
+      <c r="X55" s="123" t="n"/>
+      <c r="Y55" s="123" t="n"/>
+      <c r="Z55" s="123" t="n"/>
+      <c r="AA55" s="124" t="n"/>
     </row>
     <row r="56" ht="15" customHeight="1">
       <c r="A56" s="1" t="n"/>
@@ -29607,9 +30309,9 @@
     <mergeCell ref="B50:AA50"/>
     <mergeCell ref="B14:AA15"/>
     <mergeCell ref="B26:AA26"/>
+    <mergeCell ref="B41:AA41"/>
+    <mergeCell ref="H19:Z19"/>
     <mergeCell ref="B33:AA33"/>
-    <mergeCell ref="H19:Z19"/>
-    <mergeCell ref="B41:AA41"/>
     <mergeCell ref="B17:G17"/>
     <mergeCell ref="B4:AA4"/>
     <mergeCell ref="B35:AA35"/>

</xml_diff>

<commit_message>
Update print area margin to 105 and sync template changes
</commit_message>
<xml_diff>
--- a/static/templates/tec02-A_template.xlsx
+++ b/static/templates/tec02-A_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Paolo\diseño-afk\static\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93F0F812-236E-4D30-BE40-97F7DB213F84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{953119E7-599E-4BDC-83C6-AE64A800C09B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -578,7 +578,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -693,6 +693,19 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="25" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -702,34 +715,31 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -743,9 +753,14 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -755,24 +770,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1377,125 +1376,125 @@
     </row>
     <row r="3" spans="1:27" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2"/>
-      <c r="B3" s="57" t="s">
+      <c r="B3" s="56" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="56"/>
-      <c r="D3" s="56"/>
-      <c r="E3" s="56"/>
-      <c r="F3" s="56"/>
-      <c r="G3" s="56"/>
-      <c r="H3" s="56"/>
-      <c r="I3" s="56"/>
-      <c r="J3" s="56"/>
-      <c r="K3" s="56"/>
-      <c r="L3" s="56"/>
-      <c r="M3" s="56"/>
-      <c r="N3" s="56"/>
-      <c r="O3" s="56"/>
-      <c r="P3" s="56"/>
-      <c r="Q3" s="56"/>
-      <c r="R3" s="56"/>
-      <c r="S3" s="56"/>
-      <c r="T3" s="56"/>
-      <c r="U3" s="56"/>
-      <c r="V3" s="56"/>
-      <c r="W3" s="56"/>
-      <c r="X3" s="56"/>
-      <c r="Y3" s="56"/>
-      <c r="Z3" s="56"/>
-      <c r="AA3" s="56"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="41"/>
+      <c r="E3" s="41"/>
+      <c r="F3" s="41"/>
+      <c r="G3" s="41"/>
+      <c r="H3" s="41"/>
+      <c r="I3" s="41"/>
+      <c r="J3" s="41"/>
+      <c r="K3" s="41"/>
+      <c r="L3" s="41"/>
+      <c r="M3" s="41"/>
+      <c r="N3" s="41"/>
+      <c r="O3" s="41"/>
+      <c r="P3" s="41"/>
+      <c r="Q3" s="41"/>
+      <c r="R3" s="41"/>
+      <c r="S3" s="41"/>
+      <c r="T3" s="41"/>
+      <c r="U3" s="41"/>
+      <c r="V3" s="41"/>
+      <c r="W3" s="41"/>
+      <c r="X3" s="41"/>
+      <c r="Y3" s="41"/>
+      <c r="Z3" s="41"/>
+      <c r="AA3" s="41"/>
     </row>
     <row r="4" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="2"/>
       <c r="B4" s="61"/>
-      <c r="C4" s="56"/>
-      <c r="D4" s="56"/>
-      <c r="E4" s="56"/>
-      <c r="F4" s="56"/>
-      <c r="G4" s="56"/>
-      <c r="H4" s="56"/>
-      <c r="I4" s="56"/>
-      <c r="J4" s="56"/>
-      <c r="K4" s="56"/>
-      <c r="L4" s="56"/>
-      <c r="M4" s="56"/>
-      <c r="N4" s="56"/>
-      <c r="O4" s="56"/>
-      <c r="P4" s="56"/>
-      <c r="Q4" s="56"/>
-      <c r="R4" s="56"/>
-      <c r="S4" s="56"/>
-      <c r="T4" s="56"/>
-      <c r="U4" s="56"/>
-      <c r="V4" s="56"/>
-      <c r="W4" s="56"/>
-      <c r="X4" s="56"/>
-      <c r="Y4" s="56"/>
-      <c r="Z4" s="56"/>
-      <c r="AA4" s="56"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="41"/>
+      <c r="E4" s="41"/>
+      <c r="F4" s="41"/>
+      <c r="G4" s="41"/>
+      <c r="H4" s="41"/>
+      <c r="I4" s="41"/>
+      <c r="J4" s="41"/>
+      <c r="K4" s="41"/>
+      <c r="L4" s="41"/>
+      <c r="M4" s="41"/>
+      <c r="N4" s="41"/>
+      <c r="O4" s="41"/>
+      <c r="P4" s="41"/>
+      <c r="Q4" s="41"/>
+      <c r="R4" s="41"/>
+      <c r="S4" s="41"/>
+      <c r="T4" s="41"/>
+      <c r="U4" s="41"/>
+      <c r="V4" s="41"/>
+      <c r="W4" s="41"/>
+      <c r="X4" s="41"/>
+      <c r="Y4" s="41"/>
+      <c r="Z4" s="41"/>
+      <c r="AA4" s="41"/>
     </row>
     <row r="5" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="2"/>
       <c r="B5" s="60" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="56"/>
-      <c r="D5" s="56"/>
-      <c r="E5" s="56"/>
-      <c r="F5" s="56"/>
-      <c r="G5" s="56"/>
-      <c r="H5" s="56"/>
-      <c r="I5" s="56"/>
-      <c r="J5" s="56"/>
-      <c r="K5" s="56"/>
-      <c r="L5" s="56"/>
-      <c r="M5" s="56"/>
-      <c r="N5" s="56"/>
-      <c r="O5" s="56"/>
-      <c r="P5" s="56"/>
-      <c r="Q5" s="56"/>
-      <c r="R5" s="56"/>
-      <c r="S5" s="56"/>
-      <c r="T5" s="56"/>
-      <c r="U5" s="56"/>
-      <c r="V5" s="56"/>
-      <c r="W5" s="56"/>
-      <c r="X5" s="56"/>
-      <c r="Y5" s="56"/>
-      <c r="Z5" s="56"/>
-      <c r="AA5" s="56"/>
+      <c r="C5" s="41"/>
+      <c r="D5" s="41"/>
+      <c r="E5" s="41"/>
+      <c r="F5" s="41"/>
+      <c r="G5" s="41"/>
+      <c r="H5" s="41"/>
+      <c r="I5" s="41"/>
+      <c r="J5" s="41"/>
+      <c r="K5" s="41"/>
+      <c r="L5" s="41"/>
+      <c r="M5" s="41"/>
+      <c r="N5" s="41"/>
+      <c r="O5" s="41"/>
+      <c r="P5" s="41"/>
+      <c r="Q5" s="41"/>
+      <c r="R5" s="41"/>
+      <c r="S5" s="41"/>
+      <c r="T5" s="41"/>
+      <c r="U5" s="41"/>
+      <c r="V5" s="41"/>
+      <c r="W5" s="41"/>
+      <c r="X5" s="41"/>
+      <c r="Y5" s="41"/>
+      <c r="Z5" s="41"/>
+      <c r="AA5" s="41"/>
     </row>
     <row r="6" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="2"/>
       <c r="B6" s="58" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="56"/>
-      <c r="D6" s="56"/>
-      <c r="E6" s="56"/>
-      <c r="F6" s="56"/>
-      <c r="G6" s="56"/>
-      <c r="H6" s="56"/>
-      <c r="I6" s="56"/>
-      <c r="J6" s="56"/>
-      <c r="K6" s="56"/>
-      <c r="L6" s="56"/>
-      <c r="M6" s="56"/>
-      <c r="N6" s="56"/>
-      <c r="O6" s="56"/>
-      <c r="P6" s="56"/>
-      <c r="Q6" s="56"/>
-      <c r="R6" s="56"/>
-      <c r="S6" s="56"/>
-      <c r="T6" s="56"/>
-      <c r="U6" s="56"/>
-      <c r="V6" s="56"/>
-      <c r="W6" s="56"/>
-      <c r="X6" s="56"/>
-      <c r="Y6" s="56"/>
-      <c r="Z6" s="56"/>
-      <c r="AA6" s="56"/>
+      <c r="C6" s="41"/>
+      <c r="D6" s="41"/>
+      <c r="E6" s="41"/>
+      <c r="F6" s="41"/>
+      <c r="G6" s="41"/>
+      <c r="H6" s="41"/>
+      <c r="I6" s="41"/>
+      <c r="J6" s="41"/>
+      <c r="K6" s="41"/>
+      <c r="L6" s="41"/>
+      <c r="M6" s="41"/>
+      <c r="N6" s="41"/>
+      <c r="O6" s="41"/>
+      <c r="P6" s="41"/>
+      <c r="Q6" s="41"/>
+      <c r="R6" s="41"/>
+      <c r="S6" s="41"/>
+      <c r="T6" s="41"/>
+      <c r="U6" s="41"/>
+      <c r="V6" s="41"/>
+      <c r="W6" s="41"/>
+      <c r="X6" s="41"/>
+      <c r="Y6" s="41"/>
+      <c r="Z6" s="41"/>
+      <c r="AA6" s="41"/>
     </row>
     <row r="7" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
@@ -1594,7 +1593,7 @@
       <c r="E10" s="10"/>
       <c r="F10" s="10"/>
       <c r="G10" s="10"/>
-      <c r="H10" s="62"/>
+      <c r="H10" s="52"/>
       <c r="I10" s="53"/>
       <c r="J10" s="53"/>
       <c r="K10" s="53"/>
@@ -1654,7 +1653,7 @@
       <c r="E12" s="10"/>
       <c r="F12" s="10"/>
       <c r="G12" s="10"/>
-      <c r="H12" s="62"/>
+      <c r="H12" s="52"/>
       <c r="I12" s="53"/>
       <c r="J12" s="53"/>
       <c r="K12" s="53"/>
@@ -1708,63 +1707,63 @@
     </row>
     <row r="14" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="2"/>
-      <c r="B14" s="46" t="s">
+      <c r="B14" s="62" t="s">
         <v>2</v>
       </c>
-      <c r="C14" s="47"/>
-      <c r="D14" s="47"/>
-      <c r="E14" s="47"/>
-      <c r="F14" s="47"/>
-      <c r="G14" s="47"/>
-      <c r="H14" s="47"/>
-      <c r="I14" s="47"/>
-      <c r="J14" s="47"/>
-      <c r="K14" s="47"/>
-      <c r="L14" s="47"/>
-      <c r="M14" s="47"/>
-      <c r="N14" s="47"/>
-      <c r="O14" s="47"/>
-      <c r="P14" s="47"/>
-      <c r="Q14" s="47"/>
-      <c r="R14" s="47"/>
-      <c r="S14" s="47"/>
-      <c r="T14" s="47"/>
-      <c r="U14" s="47"/>
-      <c r="V14" s="47"/>
-      <c r="W14" s="47"/>
-      <c r="X14" s="47"/>
-      <c r="Y14" s="47"/>
-      <c r="Z14" s="47"/>
-      <c r="AA14" s="48"/>
+      <c r="C14" s="63"/>
+      <c r="D14" s="63"/>
+      <c r="E14" s="63"/>
+      <c r="F14" s="63"/>
+      <c r="G14" s="63"/>
+      <c r="H14" s="63"/>
+      <c r="I14" s="63"/>
+      <c r="J14" s="63"/>
+      <c r="K14" s="63"/>
+      <c r="L14" s="63"/>
+      <c r="M14" s="63"/>
+      <c r="N14" s="63"/>
+      <c r="O14" s="63"/>
+      <c r="P14" s="63"/>
+      <c r="Q14" s="63"/>
+      <c r="R14" s="63"/>
+      <c r="S14" s="63"/>
+      <c r="T14" s="63"/>
+      <c r="U14" s="63"/>
+      <c r="V14" s="63"/>
+      <c r="W14" s="63"/>
+      <c r="X14" s="63"/>
+      <c r="Y14" s="63"/>
+      <c r="Z14" s="63"/>
+      <c r="AA14" s="64"/>
     </row>
     <row r="15" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="2"/>
-      <c r="B15" s="49"/>
-      <c r="C15" s="50"/>
-      <c r="D15" s="50"/>
-      <c r="E15" s="50"/>
-      <c r="F15" s="50"/>
-      <c r="G15" s="50"/>
-      <c r="H15" s="50"/>
-      <c r="I15" s="50"/>
-      <c r="J15" s="50"/>
-      <c r="K15" s="50"/>
-      <c r="L15" s="50"/>
-      <c r="M15" s="50"/>
-      <c r="N15" s="50"/>
-      <c r="O15" s="50"/>
-      <c r="P15" s="50"/>
-      <c r="Q15" s="50"/>
-      <c r="R15" s="50"/>
-      <c r="S15" s="50"/>
-      <c r="T15" s="50"/>
-      <c r="U15" s="50"/>
-      <c r="V15" s="50"/>
-      <c r="W15" s="50"/>
-      <c r="X15" s="50"/>
-      <c r="Y15" s="50"/>
-      <c r="Z15" s="50"/>
-      <c r="AA15" s="51"/>
+      <c r="B15" s="65"/>
+      <c r="C15" s="66"/>
+      <c r="D15" s="66"/>
+      <c r="E15" s="66"/>
+      <c r="F15" s="66"/>
+      <c r="G15" s="66"/>
+      <c r="H15" s="66"/>
+      <c r="I15" s="66"/>
+      <c r="J15" s="66"/>
+      <c r="K15" s="66"/>
+      <c r="L15" s="66"/>
+      <c r="M15" s="66"/>
+      <c r="N15" s="66"/>
+      <c r="O15" s="66"/>
+      <c r="P15" s="66"/>
+      <c r="Q15" s="66"/>
+      <c r="R15" s="66"/>
+      <c r="S15" s="66"/>
+      <c r="T15" s="66"/>
+      <c r="U15" s="66"/>
+      <c r="V15" s="66"/>
+      <c r="W15" s="66"/>
+      <c r="X15" s="66"/>
+      <c r="Y15" s="66"/>
+      <c r="Z15" s="66"/>
+      <c r="AA15" s="67"/>
     </row>
     <row r="16" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="1"/>
@@ -1797,15 +1796,15 @@
     </row>
     <row r="17" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="1"/>
-      <c r="B17" s="55" t="s">
+      <c r="B17" s="57" t="s">
         <v>6</v>
       </c>
-      <c r="C17" s="56"/>
-      <c r="D17" s="56"/>
-      <c r="E17" s="56"/>
-      <c r="F17" s="56"/>
-      <c r="G17" s="56"/>
-      <c r="H17" s="52"/>
+      <c r="C17" s="41"/>
+      <c r="D17" s="41"/>
+      <c r="E17" s="41"/>
+      <c r="F17" s="41"/>
+      <c r="G17" s="41"/>
+      <c r="H17" s="55"/>
       <c r="I17" s="53"/>
       <c r="J17" s="53"/>
       <c r="K17" s="53"/>
@@ -1857,15 +1856,15 @@
     </row>
     <row r="19" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="1"/>
-      <c r="B19" s="55" t="s">
+      <c r="B19" s="57" t="s">
         <v>7</v>
       </c>
-      <c r="C19" s="56"/>
-      <c r="D19" s="56"/>
-      <c r="E19" s="56"/>
-      <c r="F19" s="56"/>
-      <c r="G19" s="56"/>
-      <c r="H19" s="52"/>
+      <c r="C19" s="41"/>
+      <c r="D19" s="41"/>
+      <c r="E19" s="41"/>
+      <c r="F19" s="41"/>
+      <c r="G19" s="41"/>
+      <c r="H19" s="55"/>
       <c r="I19" s="53"/>
       <c r="J19" s="53"/>
       <c r="K19" s="53"/>
@@ -1917,15 +1916,15 @@
     </row>
     <row r="21" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="1"/>
-      <c r="B21" s="55" t="s">
+      <c r="B21" s="57" t="s">
         <v>8</v>
       </c>
-      <c r="C21" s="56"/>
-      <c r="D21" s="56"/>
-      <c r="E21" s="56"/>
-      <c r="F21" s="56"/>
-      <c r="G21" s="56"/>
-      <c r="H21" s="52"/>
+      <c r="C21" s="41"/>
+      <c r="D21" s="41"/>
+      <c r="E21" s="41"/>
+      <c r="F21" s="41"/>
+      <c r="G21" s="41"/>
+      <c r="H21" s="55"/>
       <c r="I21" s="53"/>
       <c r="J21" s="53"/>
       <c r="K21" s="53"/>
@@ -1977,968 +1976,968 @@
     </row>
     <row r="23" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="1"/>
-      <c r="B23" s="63" t="s">
+      <c r="B23" s="68" t="s">
         <v>9</v>
       </c>
-      <c r="C23" s="64"/>
-      <c r="D23" s="64"/>
-      <c r="E23" s="64"/>
-      <c r="F23" s="64"/>
-      <c r="G23" s="64"/>
-      <c r="H23" s="64"/>
-      <c r="I23" s="64"/>
-      <c r="J23" s="64"/>
-      <c r="K23" s="64"/>
-      <c r="L23" s="64"/>
-      <c r="M23" s="64"/>
-      <c r="N23" s="64"/>
-      <c r="O23" s="64"/>
-      <c r="P23" s="64"/>
-      <c r="Q23" s="64"/>
-      <c r="R23" s="64"/>
-      <c r="S23" s="64"/>
-      <c r="T23" s="64"/>
-      <c r="U23" s="64"/>
-      <c r="V23" s="64"/>
-      <c r="W23" s="64"/>
-      <c r="X23" s="64"/>
-      <c r="Y23" s="64"/>
-      <c r="Z23" s="64"/>
-      <c r="AA23" s="65"/>
+      <c r="C23" s="69"/>
+      <c r="D23" s="69"/>
+      <c r="E23" s="69"/>
+      <c r="F23" s="69"/>
+      <c r="G23" s="69"/>
+      <c r="H23" s="69"/>
+      <c r="I23" s="69"/>
+      <c r="J23" s="69"/>
+      <c r="K23" s="69"/>
+      <c r="L23" s="69"/>
+      <c r="M23" s="69"/>
+      <c r="N23" s="69"/>
+      <c r="O23" s="69"/>
+      <c r="P23" s="69"/>
+      <c r="Q23" s="69"/>
+      <c r="R23" s="69"/>
+      <c r="S23" s="69"/>
+      <c r="T23" s="69"/>
+      <c r="U23" s="69"/>
+      <c r="V23" s="69"/>
+      <c r="W23" s="69"/>
+      <c r="X23" s="69"/>
+      <c r="Y23" s="69"/>
+      <c r="Z23" s="69"/>
+      <c r="AA23" s="70"/>
     </row>
     <row r="24" spans="1:27" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="1"/>
-      <c r="B24" s="40"/>
-      <c r="C24" s="41"/>
-      <c r="D24" s="41"/>
-      <c r="E24" s="41"/>
-      <c r="F24" s="41"/>
-      <c r="G24" s="41"/>
-      <c r="H24" s="41"/>
-      <c r="I24" s="41"/>
-      <c r="J24" s="41"/>
-      <c r="K24" s="41"/>
-      <c r="L24" s="41"/>
-      <c r="M24" s="41"/>
-      <c r="N24" s="41"/>
-      <c r="O24" s="41"/>
-      <c r="P24" s="41"/>
-      <c r="Q24" s="41"/>
-      <c r="R24" s="41"/>
-      <c r="S24" s="41"/>
-      <c r="T24" s="41"/>
-      <c r="U24" s="41"/>
-      <c r="V24" s="41"/>
-      <c r="W24" s="41"/>
-      <c r="X24" s="41"/>
-      <c r="Y24" s="41"/>
-      <c r="Z24" s="41"/>
-      <c r="AA24" s="42"/>
+      <c r="B24" s="45"/>
+      <c r="C24" s="46"/>
+      <c r="D24" s="46"/>
+      <c r="E24" s="46"/>
+      <c r="F24" s="46"/>
+      <c r="G24" s="46"/>
+      <c r="H24" s="46"/>
+      <c r="I24" s="46"/>
+      <c r="J24" s="46"/>
+      <c r="K24" s="46"/>
+      <c r="L24" s="46"/>
+      <c r="M24" s="46"/>
+      <c r="N24" s="46"/>
+      <c r="O24" s="46"/>
+      <c r="P24" s="46"/>
+      <c r="Q24" s="46"/>
+      <c r="R24" s="46"/>
+      <c r="S24" s="46"/>
+      <c r="T24" s="46"/>
+      <c r="U24" s="46"/>
+      <c r="V24" s="46"/>
+      <c r="W24" s="46"/>
+      <c r="X24" s="46"/>
+      <c r="Y24" s="46"/>
+      <c r="Z24" s="46"/>
+      <c r="AA24" s="47"/>
     </row>
     <row r="25" spans="1:27" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="1"/>
-      <c r="B25" s="40"/>
-      <c r="C25" s="41"/>
-      <c r="D25" s="41"/>
-      <c r="E25" s="41"/>
-      <c r="F25" s="41"/>
-      <c r="G25" s="41"/>
-      <c r="H25" s="41"/>
-      <c r="I25" s="41"/>
-      <c r="J25" s="41"/>
-      <c r="K25" s="41"/>
-      <c r="L25" s="41"/>
-      <c r="M25" s="41"/>
-      <c r="N25" s="41"/>
-      <c r="O25" s="41"/>
-      <c r="P25" s="41"/>
-      <c r="Q25" s="41"/>
-      <c r="R25" s="41"/>
-      <c r="S25" s="41"/>
-      <c r="T25" s="41"/>
-      <c r="U25" s="41"/>
-      <c r="V25" s="41"/>
-      <c r="W25" s="41"/>
-      <c r="X25" s="41"/>
-      <c r="Y25" s="41"/>
-      <c r="Z25" s="41"/>
-      <c r="AA25" s="42"/>
+      <c r="B25" s="45"/>
+      <c r="C25" s="46"/>
+      <c r="D25" s="46"/>
+      <c r="E25" s="46"/>
+      <c r="F25" s="46"/>
+      <c r="G25" s="46"/>
+      <c r="H25" s="46"/>
+      <c r="I25" s="46"/>
+      <c r="J25" s="46"/>
+      <c r="K25" s="46"/>
+      <c r="L25" s="46"/>
+      <c r="M25" s="46"/>
+      <c r="N25" s="46"/>
+      <c r="O25" s="46"/>
+      <c r="P25" s="46"/>
+      <c r="Q25" s="46"/>
+      <c r="R25" s="46"/>
+      <c r="S25" s="46"/>
+      <c r="T25" s="46"/>
+      <c r="U25" s="46"/>
+      <c r="V25" s="46"/>
+      <c r="W25" s="46"/>
+      <c r="X25" s="46"/>
+      <c r="Y25" s="46"/>
+      <c r="Z25" s="46"/>
+      <c r="AA25" s="47"/>
     </row>
     <row r="26" spans="1:27" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="1"/>
-      <c r="B26" s="40"/>
-      <c r="C26" s="41"/>
-      <c r="D26" s="41"/>
-      <c r="E26" s="41"/>
-      <c r="F26" s="41"/>
-      <c r="G26" s="41"/>
-      <c r="H26" s="41"/>
-      <c r="I26" s="41"/>
-      <c r="J26" s="41"/>
-      <c r="K26" s="41"/>
-      <c r="L26" s="41"/>
-      <c r="M26" s="41"/>
-      <c r="N26" s="41"/>
-      <c r="O26" s="41"/>
-      <c r="P26" s="41"/>
-      <c r="Q26" s="41"/>
-      <c r="R26" s="41"/>
-      <c r="S26" s="41"/>
-      <c r="T26" s="41"/>
-      <c r="U26" s="41"/>
-      <c r="V26" s="41"/>
-      <c r="W26" s="41"/>
-      <c r="X26" s="41"/>
-      <c r="Y26" s="41"/>
-      <c r="Z26" s="41"/>
-      <c r="AA26" s="42"/>
+      <c r="B26" s="45"/>
+      <c r="C26" s="46"/>
+      <c r="D26" s="46"/>
+      <c r="E26" s="46"/>
+      <c r="F26" s="46"/>
+      <c r="G26" s="46"/>
+      <c r="H26" s="46"/>
+      <c r="I26" s="46"/>
+      <c r="J26" s="46"/>
+      <c r="K26" s="46"/>
+      <c r="L26" s="46"/>
+      <c r="M26" s="46"/>
+      <c r="N26" s="46"/>
+      <c r="O26" s="46"/>
+      <c r="P26" s="46"/>
+      <c r="Q26" s="46"/>
+      <c r="R26" s="46"/>
+      <c r="S26" s="46"/>
+      <c r="T26" s="46"/>
+      <c r="U26" s="46"/>
+      <c r="V26" s="46"/>
+      <c r="W26" s="46"/>
+      <c r="X26" s="46"/>
+      <c r="Y26" s="46"/>
+      <c r="Z26" s="46"/>
+      <c r="AA26" s="47"/>
     </row>
     <row r="27" spans="1:27" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="1"/>
-      <c r="B27" s="40"/>
-      <c r="C27" s="41"/>
-      <c r="D27" s="41"/>
-      <c r="E27" s="41"/>
-      <c r="F27" s="41"/>
-      <c r="G27" s="41"/>
-      <c r="H27" s="41"/>
-      <c r="I27" s="41"/>
-      <c r="J27" s="41"/>
-      <c r="K27" s="41"/>
-      <c r="L27" s="41"/>
-      <c r="M27" s="41"/>
-      <c r="N27" s="41"/>
-      <c r="O27" s="41"/>
-      <c r="P27" s="41"/>
-      <c r="Q27" s="41"/>
-      <c r="R27" s="41"/>
-      <c r="S27" s="41"/>
-      <c r="T27" s="41"/>
-      <c r="U27" s="41"/>
-      <c r="V27" s="41"/>
-      <c r="W27" s="41"/>
-      <c r="X27" s="41"/>
-      <c r="Y27" s="41"/>
-      <c r="Z27" s="41"/>
-      <c r="AA27" s="42"/>
+      <c r="B27" s="45"/>
+      <c r="C27" s="46"/>
+      <c r="D27" s="46"/>
+      <c r="E27" s="46"/>
+      <c r="F27" s="46"/>
+      <c r="G27" s="46"/>
+      <c r="H27" s="46"/>
+      <c r="I27" s="46"/>
+      <c r="J27" s="46"/>
+      <c r="K27" s="46"/>
+      <c r="L27" s="46"/>
+      <c r="M27" s="46"/>
+      <c r="N27" s="46"/>
+      <c r="O27" s="46"/>
+      <c r="P27" s="46"/>
+      <c r="Q27" s="46"/>
+      <c r="R27" s="46"/>
+      <c r="S27" s="46"/>
+      <c r="T27" s="46"/>
+      <c r="U27" s="46"/>
+      <c r="V27" s="46"/>
+      <c r="W27" s="46"/>
+      <c r="X27" s="46"/>
+      <c r="Y27" s="46"/>
+      <c r="Z27" s="46"/>
+      <c r="AA27" s="47"/>
     </row>
     <row r="28" spans="1:27" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="1"/>
-      <c r="B28" s="40"/>
-      <c r="C28" s="41"/>
-      <c r="D28" s="41"/>
-      <c r="E28" s="41"/>
-      <c r="F28" s="41"/>
-      <c r="G28" s="41"/>
-      <c r="H28" s="41"/>
-      <c r="I28" s="41"/>
-      <c r="J28" s="41"/>
-      <c r="K28" s="41"/>
-      <c r="L28" s="41"/>
-      <c r="M28" s="41"/>
-      <c r="N28" s="41"/>
-      <c r="O28" s="41"/>
-      <c r="P28" s="41"/>
-      <c r="Q28" s="41"/>
-      <c r="R28" s="41"/>
-      <c r="S28" s="41"/>
-      <c r="T28" s="41"/>
-      <c r="U28" s="41"/>
-      <c r="V28" s="41"/>
-      <c r="W28" s="41"/>
-      <c r="X28" s="41"/>
-      <c r="Y28" s="41"/>
-      <c r="Z28" s="41"/>
-      <c r="AA28" s="42"/>
+      <c r="B28" s="45"/>
+      <c r="C28" s="46"/>
+      <c r="D28" s="46"/>
+      <c r="E28" s="46"/>
+      <c r="F28" s="46"/>
+      <c r="G28" s="46"/>
+      <c r="H28" s="46"/>
+      <c r="I28" s="46"/>
+      <c r="J28" s="46"/>
+      <c r="K28" s="46"/>
+      <c r="L28" s="46"/>
+      <c r="M28" s="46"/>
+      <c r="N28" s="46"/>
+      <c r="O28" s="46"/>
+      <c r="P28" s="46"/>
+      <c r="Q28" s="46"/>
+      <c r="R28" s="46"/>
+      <c r="S28" s="46"/>
+      <c r="T28" s="46"/>
+      <c r="U28" s="46"/>
+      <c r="V28" s="46"/>
+      <c r="W28" s="46"/>
+      <c r="X28" s="46"/>
+      <c r="Y28" s="46"/>
+      <c r="Z28" s="46"/>
+      <c r="AA28" s="47"/>
     </row>
     <row r="29" spans="1:27" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="1"/>
-      <c r="B29" s="40"/>
-      <c r="C29" s="41"/>
-      <c r="D29" s="41"/>
-      <c r="E29" s="41"/>
-      <c r="F29" s="41"/>
-      <c r="G29" s="41"/>
-      <c r="H29" s="41"/>
-      <c r="I29" s="41"/>
-      <c r="J29" s="41"/>
-      <c r="K29" s="41"/>
-      <c r="L29" s="41"/>
-      <c r="M29" s="41"/>
-      <c r="N29" s="41"/>
-      <c r="O29" s="41"/>
-      <c r="P29" s="41"/>
-      <c r="Q29" s="41"/>
-      <c r="R29" s="41"/>
-      <c r="S29" s="41"/>
-      <c r="T29" s="41"/>
-      <c r="U29" s="41"/>
-      <c r="V29" s="41"/>
-      <c r="W29" s="41"/>
-      <c r="X29" s="41"/>
-      <c r="Y29" s="41"/>
-      <c r="Z29" s="41"/>
-      <c r="AA29" s="42"/>
+      <c r="B29" s="45"/>
+      <c r="C29" s="46"/>
+      <c r="D29" s="46"/>
+      <c r="E29" s="46"/>
+      <c r="F29" s="46"/>
+      <c r="G29" s="46"/>
+      <c r="H29" s="46"/>
+      <c r="I29" s="46"/>
+      <c r="J29" s="46"/>
+      <c r="K29" s="46"/>
+      <c r="L29" s="46"/>
+      <c r="M29" s="46"/>
+      <c r="N29" s="46"/>
+      <c r="O29" s="46"/>
+      <c r="P29" s="46"/>
+      <c r="Q29" s="46"/>
+      <c r="R29" s="46"/>
+      <c r="S29" s="46"/>
+      <c r="T29" s="46"/>
+      <c r="U29" s="46"/>
+      <c r="V29" s="46"/>
+      <c r="W29" s="46"/>
+      <c r="X29" s="46"/>
+      <c r="Y29" s="46"/>
+      <c r="Z29" s="46"/>
+      <c r="AA29" s="47"/>
     </row>
     <row r="30" spans="1:27" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="1"/>
-      <c r="B30" s="40"/>
-      <c r="C30" s="41"/>
-      <c r="D30" s="41"/>
-      <c r="E30" s="41"/>
-      <c r="F30" s="41"/>
-      <c r="G30" s="41"/>
-      <c r="H30" s="41"/>
-      <c r="I30" s="41"/>
-      <c r="J30" s="41"/>
-      <c r="K30" s="41"/>
-      <c r="L30" s="41"/>
-      <c r="M30" s="41"/>
-      <c r="N30" s="41"/>
-      <c r="O30" s="41"/>
-      <c r="P30" s="41"/>
-      <c r="Q30" s="41"/>
-      <c r="R30" s="41"/>
-      <c r="S30" s="41"/>
-      <c r="T30" s="41"/>
-      <c r="U30" s="41"/>
-      <c r="V30" s="41"/>
-      <c r="W30" s="41"/>
-      <c r="X30" s="41"/>
-      <c r="Y30" s="41"/>
-      <c r="Z30" s="41"/>
-      <c r="AA30" s="42"/>
+      <c r="B30" s="45"/>
+      <c r="C30" s="46"/>
+      <c r="D30" s="46"/>
+      <c r="E30" s="46"/>
+      <c r="F30" s="46"/>
+      <c r="G30" s="46"/>
+      <c r="H30" s="46"/>
+      <c r="I30" s="46"/>
+      <c r="J30" s="46"/>
+      <c r="K30" s="46"/>
+      <c r="L30" s="46"/>
+      <c r="M30" s="46"/>
+      <c r="N30" s="46"/>
+      <c r="O30" s="46"/>
+      <c r="P30" s="46"/>
+      <c r="Q30" s="46"/>
+      <c r="R30" s="46"/>
+      <c r="S30" s="46"/>
+      <c r="T30" s="46"/>
+      <c r="U30" s="46"/>
+      <c r="V30" s="46"/>
+      <c r="W30" s="46"/>
+      <c r="X30" s="46"/>
+      <c r="Y30" s="46"/>
+      <c r="Z30" s="46"/>
+      <c r="AA30" s="47"/>
     </row>
     <row r="31" spans="1:27" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="1"/>
-      <c r="B31" s="40"/>
-      <c r="C31" s="41"/>
-      <c r="D31" s="41"/>
-      <c r="E31" s="41"/>
-      <c r="F31" s="41"/>
-      <c r="G31" s="41"/>
-      <c r="H31" s="41"/>
-      <c r="I31" s="41"/>
-      <c r="J31" s="41"/>
-      <c r="K31" s="41"/>
-      <c r="L31" s="41"/>
-      <c r="M31" s="41"/>
-      <c r="N31" s="41"/>
-      <c r="O31" s="41"/>
-      <c r="P31" s="41"/>
-      <c r="Q31" s="41"/>
-      <c r="R31" s="41"/>
-      <c r="S31" s="41"/>
-      <c r="T31" s="41"/>
-      <c r="U31" s="41"/>
-      <c r="V31" s="41"/>
-      <c r="W31" s="41"/>
-      <c r="X31" s="41"/>
-      <c r="Y31" s="41"/>
-      <c r="Z31" s="41"/>
-      <c r="AA31" s="42"/>
+      <c r="B31" s="45"/>
+      <c r="C31" s="46"/>
+      <c r="D31" s="46"/>
+      <c r="E31" s="46"/>
+      <c r="F31" s="46"/>
+      <c r="G31" s="46"/>
+      <c r="H31" s="46"/>
+      <c r="I31" s="46"/>
+      <c r="J31" s="46"/>
+      <c r="K31" s="46"/>
+      <c r="L31" s="46"/>
+      <c r="M31" s="46"/>
+      <c r="N31" s="46"/>
+      <c r="O31" s="46"/>
+      <c r="P31" s="46"/>
+      <c r="Q31" s="46"/>
+      <c r="R31" s="46"/>
+      <c r="S31" s="46"/>
+      <c r="T31" s="46"/>
+      <c r="U31" s="46"/>
+      <c r="V31" s="46"/>
+      <c r="W31" s="46"/>
+      <c r="X31" s="46"/>
+      <c r="Y31" s="46"/>
+      <c r="Z31" s="46"/>
+      <c r="AA31" s="47"/>
     </row>
     <row r="32" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="1"/>
-      <c r="B32" s="43" t="s">
+      <c r="B32" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="C32" s="44"/>
-      <c r="D32" s="44"/>
-      <c r="E32" s="44"/>
-      <c r="F32" s="44"/>
-      <c r="G32" s="44"/>
-      <c r="H32" s="44"/>
-      <c r="I32" s="44"/>
-      <c r="J32" s="44"/>
-      <c r="K32" s="44"/>
-      <c r="L32" s="44"/>
-      <c r="M32" s="44"/>
-      <c r="N32" s="44"/>
-      <c r="O32" s="44"/>
-      <c r="P32" s="44"/>
-      <c r="Q32" s="44"/>
-      <c r="R32" s="44"/>
-      <c r="S32" s="44"/>
-      <c r="T32" s="44"/>
-      <c r="U32" s="44"/>
-      <c r="V32" s="44"/>
-      <c r="W32" s="44"/>
-      <c r="X32" s="44"/>
-      <c r="Y32" s="44"/>
-      <c r="Z32" s="44"/>
-      <c r="AA32" s="45"/>
+      <c r="C32" s="43"/>
+      <c r="D32" s="43"/>
+      <c r="E32" s="43"/>
+      <c r="F32" s="43"/>
+      <c r="G32" s="43"/>
+      <c r="H32" s="43"/>
+      <c r="I32" s="43"/>
+      <c r="J32" s="43"/>
+      <c r="K32" s="43"/>
+      <c r="L32" s="43"/>
+      <c r="M32" s="43"/>
+      <c r="N32" s="43"/>
+      <c r="O32" s="43"/>
+      <c r="P32" s="43"/>
+      <c r="Q32" s="43"/>
+      <c r="R32" s="43"/>
+      <c r="S32" s="43"/>
+      <c r="T32" s="43"/>
+      <c r="U32" s="43"/>
+      <c r="V32" s="43"/>
+      <c r="W32" s="43"/>
+      <c r="X32" s="43"/>
+      <c r="Y32" s="43"/>
+      <c r="Z32" s="43"/>
+      <c r="AA32" s="44"/>
     </row>
     <row r="33" spans="1:27" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="1"/>
-      <c r="B33" s="40"/>
-      <c r="C33" s="41"/>
-      <c r="D33" s="41"/>
-      <c r="E33" s="41"/>
-      <c r="F33" s="41"/>
-      <c r="G33" s="41"/>
-      <c r="H33" s="41"/>
-      <c r="I33" s="41"/>
-      <c r="J33" s="41"/>
-      <c r="K33" s="41"/>
-      <c r="L33" s="41"/>
-      <c r="M33" s="41"/>
-      <c r="N33" s="41"/>
-      <c r="O33" s="41"/>
-      <c r="P33" s="41"/>
-      <c r="Q33" s="41"/>
-      <c r="R33" s="41"/>
-      <c r="S33" s="41"/>
-      <c r="T33" s="41"/>
-      <c r="U33" s="41"/>
-      <c r="V33" s="41"/>
-      <c r="W33" s="41"/>
-      <c r="X33" s="41"/>
-      <c r="Y33" s="41"/>
-      <c r="Z33" s="41"/>
-      <c r="AA33" s="42"/>
+      <c r="B33" s="45"/>
+      <c r="C33" s="46"/>
+      <c r="D33" s="46"/>
+      <c r="E33" s="46"/>
+      <c r="F33" s="46"/>
+      <c r="G33" s="46"/>
+      <c r="H33" s="46"/>
+      <c r="I33" s="46"/>
+      <c r="J33" s="46"/>
+      <c r="K33" s="46"/>
+      <c r="L33" s="46"/>
+      <c r="M33" s="46"/>
+      <c r="N33" s="46"/>
+      <c r="O33" s="46"/>
+      <c r="P33" s="46"/>
+      <c r="Q33" s="46"/>
+      <c r="R33" s="46"/>
+      <c r="S33" s="46"/>
+      <c r="T33" s="46"/>
+      <c r="U33" s="46"/>
+      <c r="V33" s="46"/>
+      <c r="W33" s="46"/>
+      <c r="X33" s="46"/>
+      <c r="Y33" s="46"/>
+      <c r="Z33" s="46"/>
+      <c r="AA33" s="47"/>
     </row>
     <row r="34" spans="1:27" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="1"/>
-      <c r="B34" s="40"/>
-      <c r="C34" s="41"/>
-      <c r="D34" s="41"/>
-      <c r="E34" s="41"/>
-      <c r="F34" s="41"/>
-      <c r="G34" s="41"/>
-      <c r="H34" s="41"/>
-      <c r="I34" s="41"/>
-      <c r="J34" s="41"/>
-      <c r="K34" s="41"/>
-      <c r="L34" s="41"/>
-      <c r="M34" s="41"/>
-      <c r="N34" s="41"/>
-      <c r="O34" s="41"/>
-      <c r="P34" s="41"/>
-      <c r="Q34" s="41"/>
-      <c r="R34" s="41"/>
-      <c r="S34" s="41"/>
-      <c r="T34" s="41"/>
-      <c r="U34" s="41"/>
-      <c r="V34" s="41"/>
-      <c r="W34" s="41"/>
-      <c r="X34" s="41"/>
-      <c r="Y34" s="41"/>
-      <c r="Z34" s="41"/>
-      <c r="AA34" s="42"/>
+      <c r="B34" s="45"/>
+      <c r="C34" s="46"/>
+      <c r="D34" s="46"/>
+      <c r="E34" s="46"/>
+      <c r="F34" s="46"/>
+      <c r="G34" s="46"/>
+      <c r="H34" s="46"/>
+      <c r="I34" s="46"/>
+      <c r="J34" s="46"/>
+      <c r="K34" s="46"/>
+      <c r="L34" s="46"/>
+      <c r="M34" s="46"/>
+      <c r="N34" s="46"/>
+      <c r="O34" s="46"/>
+      <c r="P34" s="46"/>
+      <c r="Q34" s="46"/>
+      <c r="R34" s="46"/>
+      <c r="S34" s="46"/>
+      <c r="T34" s="46"/>
+      <c r="U34" s="46"/>
+      <c r="V34" s="46"/>
+      <c r="W34" s="46"/>
+      <c r="X34" s="46"/>
+      <c r="Y34" s="46"/>
+      <c r="Z34" s="46"/>
+      <c r="AA34" s="47"/>
     </row>
     <row r="35" spans="1:27" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="1"/>
-      <c r="B35" s="40"/>
-      <c r="C35" s="41"/>
-      <c r="D35" s="41"/>
-      <c r="E35" s="41"/>
-      <c r="F35" s="41"/>
-      <c r="G35" s="41"/>
-      <c r="H35" s="41"/>
-      <c r="I35" s="41"/>
-      <c r="J35" s="41"/>
-      <c r="K35" s="41"/>
-      <c r="L35" s="41"/>
-      <c r="M35" s="41"/>
-      <c r="N35" s="41"/>
-      <c r="O35" s="41"/>
-      <c r="P35" s="41"/>
-      <c r="Q35" s="41"/>
-      <c r="R35" s="41"/>
-      <c r="S35" s="41"/>
-      <c r="T35" s="41"/>
-      <c r="U35" s="41"/>
-      <c r="V35" s="41"/>
-      <c r="W35" s="41"/>
-      <c r="X35" s="41"/>
-      <c r="Y35" s="41"/>
-      <c r="Z35" s="41"/>
-      <c r="AA35" s="42"/>
+      <c r="B35" s="45"/>
+      <c r="C35" s="46"/>
+      <c r="D35" s="46"/>
+      <c r="E35" s="46"/>
+      <c r="F35" s="46"/>
+      <c r="G35" s="46"/>
+      <c r="H35" s="46"/>
+      <c r="I35" s="46"/>
+      <c r="J35" s="46"/>
+      <c r="K35" s="46"/>
+      <c r="L35" s="46"/>
+      <c r="M35" s="46"/>
+      <c r="N35" s="46"/>
+      <c r="O35" s="46"/>
+      <c r="P35" s="46"/>
+      <c r="Q35" s="46"/>
+      <c r="R35" s="46"/>
+      <c r="S35" s="46"/>
+      <c r="T35" s="46"/>
+      <c r="U35" s="46"/>
+      <c r="V35" s="46"/>
+      <c r="W35" s="46"/>
+      <c r="X35" s="46"/>
+      <c r="Y35" s="46"/>
+      <c r="Z35" s="46"/>
+      <c r="AA35" s="47"/>
     </row>
     <row r="36" spans="1:27" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="1"/>
-      <c r="B36" s="40"/>
-      <c r="C36" s="41"/>
-      <c r="D36" s="41"/>
-      <c r="E36" s="41"/>
-      <c r="F36" s="41"/>
-      <c r="G36" s="41"/>
-      <c r="H36" s="41"/>
-      <c r="I36" s="41"/>
-      <c r="J36" s="41"/>
-      <c r="K36" s="41"/>
-      <c r="L36" s="41"/>
-      <c r="M36" s="41"/>
-      <c r="N36" s="41"/>
-      <c r="O36" s="41"/>
-      <c r="P36" s="41"/>
-      <c r="Q36" s="41"/>
-      <c r="R36" s="41"/>
-      <c r="S36" s="41"/>
-      <c r="T36" s="41"/>
-      <c r="U36" s="41"/>
-      <c r="V36" s="41"/>
-      <c r="W36" s="41"/>
-      <c r="X36" s="41"/>
-      <c r="Y36" s="41"/>
-      <c r="Z36" s="41"/>
-      <c r="AA36" s="42"/>
+      <c r="B36" s="45"/>
+      <c r="C36" s="46"/>
+      <c r="D36" s="46"/>
+      <c r="E36" s="46"/>
+      <c r="F36" s="46"/>
+      <c r="G36" s="46"/>
+      <c r="H36" s="46"/>
+      <c r="I36" s="46"/>
+      <c r="J36" s="46"/>
+      <c r="K36" s="46"/>
+      <c r="L36" s="46"/>
+      <c r="M36" s="46"/>
+      <c r="N36" s="46"/>
+      <c r="O36" s="46"/>
+      <c r="P36" s="46"/>
+      <c r="Q36" s="46"/>
+      <c r="R36" s="46"/>
+      <c r="S36" s="46"/>
+      <c r="T36" s="46"/>
+      <c r="U36" s="46"/>
+      <c r="V36" s="46"/>
+      <c r="W36" s="46"/>
+      <c r="X36" s="46"/>
+      <c r="Y36" s="46"/>
+      <c r="Z36" s="46"/>
+      <c r="AA36" s="47"/>
     </row>
     <row r="37" spans="1:27" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="1"/>
-      <c r="B37" s="40"/>
-      <c r="C37" s="41"/>
-      <c r="D37" s="41"/>
-      <c r="E37" s="41"/>
-      <c r="F37" s="41"/>
-      <c r="G37" s="41"/>
-      <c r="H37" s="41"/>
-      <c r="I37" s="41"/>
-      <c r="J37" s="41"/>
-      <c r="K37" s="41"/>
-      <c r="L37" s="41"/>
-      <c r="M37" s="41"/>
-      <c r="N37" s="41"/>
-      <c r="O37" s="41"/>
-      <c r="P37" s="41"/>
-      <c r="Q37" s="41"/>
-      <c r="R37" s="41"/>
-      <c r="S37" s="41"/>
-      <c r="T37" s="41"/>
-      <c r="U37" s="41"/>
-      <c r="V37" s="41"/>
-      <c r="W37" s="41"/>
-      <c r="X37" s="41"/>
-      <c r="Y37" s="41"/>
-      <c r="Z37" s="41"/>
-      <c r="AA37" s="42"/>
+      <c r="B37" s="45"/>
+      <c r="C37" s="46"/>
+      <c r="D37" s="46"/>
+      <c r="E37" s="46"/>
+      <c r="F37" s="46"/>
+      <c r="G37" s="46"/>
+      <c r="H37" s="46"/>
+      <c r="I37" s="46"/>
+      <c r="J37" s="46"/>
+      <c r="K37" s="46"/>
+      <c r="L37" s="46"/>
+      <c r="M37" s="46"/>
+      <c r="N37" s="46"/>
+      <c r="O37" s="46"/>
+      <c r="P37" s="46"/>
+      <c r="Q37" s="46"/>
+      <c r="R37" s="46"/>
+      <c r="S37" s="46"/>
+      <c r="T37" s="46"/>
+      <c r="U37" s="46"/>
+      <c r="V37" s="46"/>
+      <c r="W37" s="46"/>
+      <c r="X37" s="46"/>
+      <c r="Y37" s="46"/>
+      <c r="Z37" s="46"/>
+      <c r="AA37" s="47"/>
     </row>
     <row r="38" spans="1:27" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="1"/>
-      <c r="B38" s="40"/>
-      <c r="C38" s="41"/>
-      <c r="D38" s="41"/>
-      <c r="E38" s="41"/>
-      <c r="F38" s="41"/>
-      <c r="G38" s="41"/>
-      <c r="H38" s="41"/>
-      <c r="I38" s="41"/>
-      <c r="J38" s="41"/>
-      <c r="K38" s="41"/>
-      <c r="L38" s="41"/>
-      <c r="M38" s="41"/>
-      <c r="N38" s="41"/>
-      <c r="O38" s="41"/>
-      <c r="P38" s="41"/>
-      <c r="Q38" s="41"/>
-      <c r="R38" s="41"/>
-      <c r="S38" s="41"/>
-      <c r="T38" s="41"/>
-      <c r="U38" s="41"/>
-      <c r="V38" s="41"/>
-      <c r="W38" s="41"/>
-      <c r="X38" s="41"/>
-      <c r="Y38" s="41"/>
-      <c r="Z38" s="41"/>
-      <c r="AA38" s="42"/>
+      <c r="B38" s="45"/>
+      <c r="C38" s="46"/>
+      <c r="D38" s="46"/>
+      <c r="E38" s="46"/>
+      <c r="F38" s="46"/>
+      <c r="G38" s="46"/>
+      <c r="H38" s="46"/>
+      <c r="I38" s="46"/>
+      <c r="J38" s="46"/>
+      <c r="K38" s="46"/>
+      <c r="L38" s="46"/>
+      <c r="M38" s="46"/>
+      <c r="N38" s="46"/>
+      <c r="O38" s="46"/>
+      <c r="P38" s="46"/>
+      <c r="Q38" s="46"/>
+      <c r="R38" s="46"/>
+      <c r="S38" s="46"/>
+      <c r="T38" s="46"/>
+      <c r="U38" s="46"/>
+      <c r="V38" s="46"/>
+      <c r="W38" s="46"/>
+      <c r="X38" s="46"/>
+      <c r="Y38" s="46"/>
+      <c r="Z38" s="46"/>
+      <c r="AA38" s="47"/>
     </row>
     <row r="39" spans="1:27" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="1"/>
-      <c r="B39" s="40"/>
-      <c r="C39" s="41"/>
-      <c r="D39" s="41"/>
-      <c r="E39" s="41"/>
-      <c r="F39" s="41"/>
-      <c r="G39" s="41"/>
-      <c r="H39" s="41"/>
-      <c r="I39" s="41"/>
-      <c r="J39" s="41"/>
-      <c r="K39" s="41"/>
-      <c r="L39" s="41"/>
-      <c r="M39" s="41"/>
-      <c r="N39" s="41"/>
-      <c r="O39" s="41"/>
-      <c r="P39" s="41"/>
-      <c r="Q39" s="41"/>
-      <c r="R39" s="41"/>
-      <c r="S39" s="41"/>
-      <c r="T39" s="41"/>
-      <c r="U39" s="41"/>
-      <c r="V39" s="41"/>
-      <c r="W39" s="41"/>
-      <c r="X39" s="41"/>
-      <c r="Y39" s="41"/>
-      <c r="Z39" s="41"/>
-      <c r="AA39" s="42"/>
+      <c r="B39" s="45"/>
+      <c r="C39" s="46"/>
+      <c r="D39" s="46"/>
+      <c r="E39" s="46"/>
+      <c r="F39" s="46"/>
+      <c r="G39" s="46"/>
+      <c r="H39" s="46"/>
+      <c r="I39" s="46"/>
+      <c r="J39" s="46"/>
+      <c r="K39" s="46"/>
+      <c r="L39" s="46"/>
+      <c r="M39" s="46"/>
+      <c r="N39" s="46"/>
+      <c r="O39" s="46"/>
+      <c r="P39" s="46"/>
+      <c r="Q39" s="46"/>
+      <c r="R39" s="46"/>
+      <c r="S39" s="46"/>
+      <c r="T39" s="46"/>
+      <c r="U39" s="46"/>
+      <c r="V39" s="46"/>
+      <c r="W39" s="46"/>
+      <c r="X39" s="46"/>
+      <c r="Y39" s="46"/>
+      <c r="Z39" s="46"/>
+      <c r="AA39" s="47"/>
     </row>
     <row r="40" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="1"/>
-      <c r="B40" s="43" t="s">
+      <c r="B40" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="C40" s="44"/>
-      <c r="D40" s="44"/>
-      <c r="E40" s="44"/>
-      <c r="F40" s="44"/>
-      <c r="G40" s="44"/>
-      <c r="H40" s="44"/>
-      <c r="I40" s="44"/>
-      <c r="J40" s="44"/>
-      <c r="K40" s="44"/>
-      <c r="L40" s="44"/>
-      <c r="M40" s="44"/>
-      <c r="N40" s="44"/>
-      <c r="O40" s="44"/>
-      <c r="P40" s="44"/>
-      <c r="Q40" s="44"/>
-      <c r="R40" s="44"/>
-      <c r="S40" s="44"/>
-      <c r="T40" s="44"/>
-      <c r="U40" s="44"/>
-      <c r="V40" s="44"/>
-      <c r="W40" s="44"/>
-      <c r="X40" s="44"/>
-      <c r="Y40" s="44"/>
-      <c r="Z40" s="44"/>
-      <c r="AA40" s="45"/>
+      <c r="C40" s="43"/>
+      <c r="D40" s="43"/>
+      <c r="E40" s="43"/>
+      <c r="F40" s="43"/>
+      <c r="G40" s="43"/>
+      <c r="H40" s="43"/>
+      <c r="I40" s="43"/>
+      <c r="J40" s="43"/>
+      <c r="K40" s="43"/>
+      <c r="L40" s="43"/>
+      <c r="M40" s="43"/>
+      <c r="N40" s="43"/>
+      <c r="O40" s="43"/>
+      <c r="P40" s="43"/>
+      <c r="Q40" s="43"/>
+      <c r="R40" s="43"/>
+      <c r="S40" s="43"/>
+      <c r="T40" s="43"/>
+      <c r="U40" s="43"/>
+      <c r="V40" s="43"/>
+      <c r="W40" s="43"/>
+      <c r="X40" s="43"/>
+      <c r="Y40" s="43"/>
+      <c r="Z40" s="43"/>
+      <c r="AA40" s="44"/>
     </row>
     <row r="41" spans="1:27" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="1"/>
-      <c r="B41" s="40"/>
-      <c r="C41" s="41"/>
-      <c r="D41" s="41"/>
-      <c r="E41" s="41"/>
-      <c r="F41" s="41"/>
-      <c r="G41" s="41"/>
-      <c r="H41" s="41"/>
-      <c r="I41" s="41"/>
-      <c r="J41" s="41"/>
-      <c r="K41" s="41"/>
-      <c r="L41" s="41"/>
-      <c r="M41" s="41"/>
-      <c r="N41" s="41"/>
-      <c r="O41" s="41"/>
-      <c r="P41" s="41"/>
-      <c r="Q41" s="41"/>
-      <c r="R41" s="41"/>
-      <c r="S41" s="41"/>
-      <c r="T41" s="41"/>
-      <c r="U41" s="41"/>
-      <c r="V41" s="41"/>
-      <c r="W41" s="41"/>
-      <c r="X41" s="41"/>
-      <c r="Y41" s="41"/>
-      <c r="Z41" s="41"/>
-      <c r="AA41" s="42"/>
+      <c r="B41" s="45"/>
+      <c r="C41" s="46"/>
+      <c r="D41" s="46"/>
+      <c r="E41" s="46"/>
+      <c r="F41" s="46"/>
+      <c r="G41" s="46"/>
+      <c r="H41" s="46"/>
+      <c r="I41" s="46"/>
+      <c r="J41" s="46"/>
+      <c r="K41" s="46"/>
+      <c r="L41" s="46"/>
+      <c r="M41" s="46"/>
+      <c r="N41" s="46"/>
+      <c r="O41" s="46"/>
+      <c r="P41" s="46"/>
+      <c r="Q41" s="46"/>
+      <c r="R41" s="46"/>
+      <c r="S41" s="46"/>
+      <c r="T41" s="46"/>
+      <c r="U41" s="46"/>
+      <c r="V41" s="46"/>
+      <c r="W41" s="46"/>
+      <c r="X41" s="46"/>
+      <c r="Y41" s="46"/>
+      <c r="Z41" s="46"/>
+      <c r="AA41" s="47"/>
     </row>
     <row r="42" spans="1:27" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="1"/>
-      <c r="B42" s="40"/>
-      <c r="C42" s="41"/>
-      <c r="D42" s="41"/>
-      <c r="E42" s="41"/>
-      <c r="F42" s="41"/>
-      <c r="G42" s="41"/>
-      <c r="H42" s="41"/>
-      <c r="I42" s="41"/>
-      <c r="J42" s="41"/>
-      <c r="K42" s="41"/>
-      <c r="L42" s="41"/>
-      <c r="M42" s="41"/>
-      <c r="N42" s="41"/>
-      <c r="O42" s="41"/>
-      <c r="P42" s="41"/>
-      <c r="Q42" s="41"/>
-      <c r="R42" s="41"/>
-      <c r="S42" s="41"/>
-      <c r="T42" s="41"/>
-      <c r="U42" s="41"/>
-      <c r="V42" s="41"/>
-      <c r="W42" s="41"/>
-      <c r="X42" s="41"/>
-      <c r="Y42" s="41"/>
-      <c r="Z42" s="41"/>
-      <c r="AA42" s="42"/>
+      <c r="B42" s="45"/>
+      <c r="C42" s="46"/>
+      <c r="D42" s="46"/>
+      <c r="E42" s="46"/>
+      <c r="F42" s="46"/>
+      <c r="G42" s="46"/>
+      <c r="H42" s="46"/>
+      <c r="I42" s="46"/>
+      <c r="J42" s="46"/>
+      <c r="K42" s="46"/>
+      <c r="L42" s="46"/>
+      <c r="M42" s="46"/>
+      <c r="N42" s="46"/>
+      <c r="O42" s="46"/>
+      <c r="P42" s="46"/>
+      <c r="Q42" s="46"/>
+      <c r="R42" s="46"/>
+      <c r="S42" s="46"/>
+      <c r="T42" s="46"/>
+      <c r="U42" s="46"/>
+      <c r="V42" s="46"/>
+      <c r="W42" s="46"/>
+      <c r="X42" s="46"/>
+      <c r="Y42" s="46"/>
+      <c r="Z42" s="46"/>
+      <c r="AA42" s="47"/>
     </row>
     <row r="43" spans="1:27" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="1"/>
-      <c r="B43" s="40"/>
-      <c r="C43" s="41"/>
-      <c r="D43" s="41"/>
-      <c r="E43" s="41"/>
-      <c r="F43" s="41"/>
-      <c r="G43" s="41"/>
-      <c r="H43" s="41"/>
-      <c r="I43" s="41"/>
-      <c r="J43" s="41"/>
-      <c r="K43" s="41"/>
-      <c r="L43" s="41"/>
-      <c r="M43" s="41"/>
-      <c r="N43" s="41"/>
-      <c r="O43" s="41"/>
-      <c r="P43" s="41"/>
-      <c r="Q43" s="41"/>
-      <c r="R43" s="41"/>
-      <c r="S43" s="41"/>
-      <c r="T43" s="41"/>
-      <c r="U43" s="41"/>
-      <c r="V43" s="41"/>
-      <c r="W43" s="41"/>
-      <c r="X43" s="41"/>
-      <c r="Y43" s="41"/>
-      <c r="Z43" s="41"/>
-      <c r="AA43" s="42"/>
+      <c r="B43" s="45"/>
+      <c r="C43" s="46"/>
+      <c r="D43" s="46"/>
+      <c r="E43" s="46"/>
+      <c r="F43" s="46"/>
+      <c r="G43" s="46"/>
+      <c r="H43" s="46"/>
+      <c r="I43" s="46"/>
+      <c r="J43" s="46"/>
+      <c r="K43" s="46"/>
+      <c r="L43" s="46"/>
+      <c r="M43" s="46"/>
+      <c r="N43" s="46"/>
+      <c r="O43" s="46"/>
+      <c r="P43" s="46"/>
+      <c r="Q43" s="46"/>
+      <c r="R43" s="46"/>
+      <c r="S43" s="46"/>
+      <c r="T43" s="46"/>
+      <c r="U43" s="46"/>
+      <c r="V43" s="46"/>
+      <c r="W43" s="46"/>
+      <c r="X43" s="46"/>
+      <c r="Y43" s="46"/>
+      <c r="Z43" s="46"/>
+      <c r="AA43" s="47"/>
     </row>
     <row r="44" spans="1:27" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="1"/>
-      <c r="B44" s="40"/>
-      <c r="C44" s="41"/>
-      <c r="D44" s="41"/>
-      <c r="E44" s="41"/>
-      <c r="F44" s="41"/>
-      <c r="G44" s="41"/>
-      <c r="H44" s="41"/>
-      <c r="I44" s="41"/>
-      <c r="J44" s="41"/>
-      <c r="K44" s="41"/>
-      <c r="L44" s="41"/>
-      <c r="M44" s="41"/>
-      <c r="N44" s="41"/>
-      <c r="O44" s="41"/>
-      <c r="P44" s="41"/>
-      <c r="Q44" s="41"/>
-      <c r="R44" s="41"/>
-      <c r="S44" s="41"/>
-      <c r="T44" s="41"/>
-      <c r="U44" s="41"/>
-      <c r="V44" s="41"/>
-      <c r="W44" s="41"/>
-      <c r="X44" s="41"/>
-      <c r="Y44" s="41"/>
-      <c r="Z44" s="41"/>
-      <c r="AA44" s="42"/>
+      <c r="B44" s="45"/>
+      <c r="C44" s="46"/>
+      <c r="D44" s="46"/>
+      <c r="E44" s="46"/>
+      <c r="F44" s="46"/>
+      <c r="G44" s="46"/>
+      <c r="H44" s="46"/>
+      <c r="I44" s="46"/>
+      <c r="J44" s="46"/>
+      <c r="K44" s="46"/>
+      <c r="L44" s="46"/>
+      <c r="M44" s="46"/>
+      <c r="N44" s="46"/>
+      <c r="O44" s="46"/>
+      <c r="P44" s="46"/>
+      <c r="Q44" s="46"/>
+      <c r="R44" s="46"/>
+      <c r="S44" s="46"/>
+      <c r="T44" s="46"/>
+      <c r="U44" s="46"/>
+      <c r="V44" s="46"/>
+      <c r="W44" s="46"/>
+      <c r="X44" s="46"/>
+      <c r="Y44" s="46"/>
+      <c r="Z44" s="46"/>
+      <c r="AA44" s="47"/>
     </row>
     <row r="45" spans="1:27" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="1"/>
-      <c r="B45" s="40"/>
-      <c r="C45" s="41"/>
-      <c r="D45" s="41"/>
-      <c r="E45" s="41"/>
-      <c r="F45" s="41"/>
-      <c r="G45" s="41"/>
-      <c r="H45" s="41"/>
-      <c r="I45" s="41"/>
-      <c r="J45" s="41"/>
-      <c r="K45" s="41"/>
-      <c r="L45" s="41"/>
-      <c r="M45" s="41"/>
-      <c r="N45" s="41"/>
-      <c r="O45" s="41"/>
-      <c r="P45" s="41"/>
-      <c r="Q45" s="41"/>
-      <c r="R45" s="41"/>
-      <c r="S45" s="41"/>
-      <c r="T45" s="41"/>
-      <c r="U45" s="41"/>
-      <c r="V45" s="41"/>
-      <c r="W45" s="41"/>
-      <c r="X45" s="41"/>
-      <c r="Y45" s="41"/>
-      <c r="Z45" s="41"/>
-      <c r="AA45" s="42"/>
+      <c r="B45" s="45"/>
+      <c r="C45" s="46"/>
+      <c r="D45" s="46"/>
+      <c r="E45" s="46"/>
+      <c r="F45" s="46"/>
+      <c r="G45" s="46"/>
+      <c r="H45" s="46"/>
+      <c r="I45" s="46"/>
+      <c r="J45" s="46"/>
+      <c r="K45" s="46"/>
+      <c r="L45" s="46"/>
+      <c r="M45" s="46"/>
+      <c r="N45" s="46"/>
+      <c r="O45" s="46"/>
+      <c r="P45" s="46"/>
+      <c r="Q45" s="46"/>
+      <c r="R45" s="46"/>
+      <c r="S45" s="46"/>
+      <c r="T45" s="46"/>
+      <c r="U45" s="46"/>
+      <c r="V45" s="46"/>
+      <c r="W45" s="46"/>
+      <c r="X45" s="46"/>
+      <c r="Y45" s="46"/>
+      <c r="Z45" s="46"/>
+      <c r="AA45" s="47"/>
     </row>
     <row r="46" spans="1:27" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="1"/>
-      <c r="B46" s="40"/>
-      <c r="C46" s="41"/>
-      <c r="D46" s="41"/>
-      <c r="E46" s="41"/>
-      <c r="F46" s="41"/>
-      <c r="G46" s="41"/>
-      <c r="H46" s="41"/>
-      <c r="I46" s="41"/>
-      <c r="J46" s="41"/>
-      <c r="K46" s="41"/>
-      <c r="L46" s="41"/>
-      <c r="M46" s="41"/>
-      <c r="N46" s="41"/>
-      <c r="O46" s="41"/>
-      <c r="P46" s="41"/>
-      <c r="Q46" s="41"/>
-      <c r="R46" s="41"/>
-      <c r="S46" s="41"/>
-      <c r="T46" s="41"/>
-      <c r="U46" s="41"/>
-      <c r="V46" s="41"/>
-      <c r="W46" s="41"/>
-      <c r="X46" s="41"/>
-      <c r="Y46" s="41"/>
-      <c r="Z46" s="41"/>
-      <c r="AA46" s="42"/>
+      <c r="B46" s="45"/>
+      <c r="C46" s="46"/>
+      <c r="D46" s="46"/>
+      <c r="E46" s="46"/>
+      <c r="F46" s="46"/>
+      <c r="G46" s="46"/>
+      <c r="H46" s="46"/>
+      <c r="I46" s="46"/>
+      <c r="J46" s="46"/>
+      <c r="K46" s="46"/>
+      <c r="L46" s="46"/>
+      <c r="M46" s="46"/>
+      <c r="N46" s="46"/>
+      <c r="O46" s="46"/>
+      <c r="P46" s="46"/>
+      <c r="Q46" s="46"/>
+      <c r="R46" s="46"/>
+      <c r="S46" s="46"/>
+      <c r="T46" s="46"/>
+      <c r="U46" s="46"/>
+      <c r="V46" s="46"/>
+      <c r="W46" s="46"/>
+      <c r="X46" s="46"/>
+      <c r="Y46" s="46"/>
+      <c r="Z46" s="46"/>
+      <c r="AA46" s="47"/>
     </row>
     <row r="47" spans="1:27" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="1"/>
-      <c r="B47" s="40"/>
-      <c r="C47" s="41"/>
-      <c r="D47" s="41"/>
-      <c r="E47" s="41"/>
-      <c r="F47" s="41"/>
-      <c r="G47" s="41"/>
-      <c r="H47" s="41"/>
-      <c r="I47" s="41"/>
-      <c r="J47" s="41"/>
-      <c r="K47" s="41"/>
-      <c r="L47" s="41"/>
-      <c r="M47" s="41"/>
-      <c r="N47" s="41"/>
-      <c r="O47" s="41"/>
-      <c r="P47" s="41"/>
-      <c r="Q47" s="41"/>
-      <c r="R47" s="41"/>
-      <c r="S47" s="41"/>
-      <c r="T47" s="41"/>
-      <c r="U47" s="41"/>
-      <c r="V47" s="41"/>
-      <c r="W47" s="41"/>
-      <c r="X47" s="41"/>
-      <c r="Y47" s="41"/>
-      <c r="Z47" s="41"/>
-      <c r="AA47" s="42"/>
+      <c r="B47" s="45"/>
+      <c r="C47" s="46"/>
+      <c r="D47" s="46"/>
+      <c r="E47" s="46"/>
+      <c r="F47" s="46"/>
+      <c r="G47" s="46"/>
+      <c r="H47" s="46"/>
+      <c r="I47" s="46"/>
+      <c r="J47" s="46"/>
+      <c r="K47" s="46"/>
+      <c r="L47" s="46"/>
+      <c r="M47" s="46"/>
+      <c r="N47" s="46"/>
+      <c r="O47" s="46"/>
+      <c r="P47" s="46"/>
+      <c r="Q47" s="46"/>
+      <c r="R47" s="46"/>
+      <c r="S47" s="46"/>
+      <c r="T47" s="46"/>
+      <c r="U47" s="46"/>
+      <c r="V47" s="46"/>
+      <c r="W47" s="46"/>
+      <c r="X47" s="46"/>
+      <c r="Y47" s="46"/>
+      <c r="Z47" s="46"/>
+      <c r="AA47" s="47"/>
     </row>
     <row r="48" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" s="1"/>
-      <c r="B48" s="69" t="s">
+      <c r="B48" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="C48" s="70"/>
-      <c r="D48" s="70"/>
-      <c r="E48" s="70"/>
-      <c r="F48" s="70"/>
-      <c r="G48" s="70"/>
-      <c r="H48" s="70"/>
-      <c r="I48" s="70"/>
-      <c r="J48" s="70"/>
-      <c r="K48" s="70"/>
-      <c r="L48" s="70"/>
-      <c r="M48" s="70"/>
-      <c r="N48" s="70"/>
-      <c r="O48" s="70"/>
-      <c r="P48" s="70"/>
-      <c r="Q48" s="70"/>
-      <c r="R48" s="70"/>
-      <c r="S48" s="70"/>
-      <c r="T48" s="70"/>
-      <c r="U48" s="70"/>
-      <c r="V48" s="70"/>
-      <c r="W48" s="70"/>
-      <c r="X48" s="70"/>
-      <c r="Y48" s="70"/>
-      <c r="Z48" s="70"/>
-      <c r="AA48" s="71"/>
+      <c r="C48" s="49"/>
+      <c r="D48" s="49"/>
+      <c r="E48" s="49"/>
+      <c r="F48" s="49"/>
+      <c r="G48" s="49"/>
+      <c r="H48" s="49"/>
+      <c r="I48" s="49"/>
+      <c r="J48" s="49"/>
+      <c r="K48" s="49"/>
+      <c r="L48" s="49"/>
+      <c r="M48" s="49"/>
+      <c r="N48" s="49"/>
+      <c r="O48" s="49"/>
+      <c r="P48" s="49"/>
+      <c r="Q48" s="49"/>
+      <c r="R48" s="49"/>
+      <c r="S48" s="49"/>
+      <c r="T48" s="49"/>
+      <c r="U48" s="49"/>
+      <c r="V48" s="49"/>
+      <c r="W48" s="49"/>
+      <c r="X48" s="49"/>
+      <c r="Y48" s="49"/>
+      <c r="Z48" s="49"/>
+      <c r="AA48" s="50"/>
     </row>
     <row r="49" spans="1:27" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" s="30"/>
-      <c r="B49" s="40"/>
-      <c r="C49" s="41"/>
-      <c r="D49" s="41"/>
-      <c r="E49" s="41"/>
-      <c r="F49" s="41"/>
-      <c r="G49" s="41"/>
-      <c r="H49" s="41"/>
-      <c r="I49" s="41"/>
-      <c r="J49" s="41"/>
-      <c r="K49" s="41"/>
-      <c r="L49" s="41"/>
-      <c r="M49" s="41"/>
-      <c r="N49" s="41"/>
-      <c r="O49" s="41"/>
-      <c r="P49" s="41"/>
-      <c r="Q49" s="41"/>
-      <c r="R49" s="41"/>
-      <c r="S49" s="41"/>
-      <c r="T49" s="41"/>
-      <c r="U49" s="41"/>
-      <c r="V49" s="41"/>
-      <c r="W49" s="41"/>
-      <c r="X49" s="41"/>
-      <c r="Y49" s="41"/>
-      <c r="Z49" s="41"/>
-      <c r="AA49" s="42"/>
+      <c r="B49" s="45"/>
+      <c r="C49" s="46"/>
+      <c r="D49" s="46"/>
+      <c r="E49" s="46"/>
+      <c r="F49" s="46"/>
+      <c r="G49" s="46"/>
+      <c r="H49" s="46"/>
+      <c r="I49" s="46"/>
+      <c r="J49" s="46"/>
+      <c r="K49" s="46"/>
+      <c r="L49" s="46"/>
+      <c r="M49" s="46"/>
+      <c r="N49" s="46"/>
+      <c r="O49" s="46"/>
+      <c r="P49" s="46"/>
+      <c r="Q49" s="46"/>
+      <c r="R49" s="46"/>
+      <c r="S49" s="46"/>
+      <c r="T49" s="46"/>
+      <c r="U49" s="46"/>
+      <c r="V49" s="46"/>
+      <c r="W49" s="46"/>
+      <c r="X49" s="46"/>
+      <c r="Y49" s="46"/>
+      <c r="Z49" s="46"/>
+      <c r="AA49" s="47"/>
     </row>
     <row r="50" spans="1:27" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50" s="30"/>
-      <c r="B50" s="40"/>
-      <c r="C50" s="41"/>
-      <c r="D50" s="41"/>
-      <c r="E50" s="41"/>
-      <c r="F50" s="41"/>
-      <c r="G50" s="41"/>
-      <c r="H50" s="41"/>
-      <c r="I50" s="41"/>
-      <c r="J50" s="41"/>
-      <c r="K50" s="41"/>
-      <c r="L50" s="41"/>
-      <c r="M50" s="41"/>
-      <c r="N50" s="41"/>
-      <c r="O50" s="41"/>
-      <c r="P50" s="41"/>
-      <c r="Q50" s="41"/>
-      <c r="R50" s="41"/>
-      <c r="S50" s="41"/>
-      <c r="T50" s="41"/>
-      <c r="U50" s="41"/>
-      <c r="V50" s="41"/>
-      <c r="W50" s="41"/>
-      <c r="X50" s="41"/>
-      <c r="Y50" s="41"/>
-      <c r="Z50" s="41"/>
-      <c r="AA50" s="42"/>
+      <c r="B50" s="45"/>
+      <c r="C50" s="46"/>
+      <c r="D50" s="46"/>
+      <c r="E50" s="46"/>
+      <c r="F50" s="46"/>
+      <c r="G50" s="46"/>
+      <c r="H50" s="46"/>
+      <c r="I50" s="46"/>
+      <c r="J50" s="46"/>
+      <c r="K50" s="46"/>
+      <c r="L50" s="46"/>
+      <c r="M50" s="46"/>
+      <c r="N50" s="46"/>
+      <c r="O50" s="46"/>
+      <c r="P50" s="46"/>
+      <c r="Q50" s="46"/>
+      <c r="R50" s="46"/>
+      <c r="S50" s="46"/>
+      <c r="T50" s="46"/>
+      <c r="U50" s="46"/>
+      <c r="V50" s="46"/>
+      <c r="W50" s="46"/>
+      <c r="X50" s="46"/>
+      <c r="Y50" s="46"/>
+      <c r="Z50" s="46"/>
+      <c r="AA50" s="47"/>
     </row>
     <row r="51" spans="1:27" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51" s="30"/>
-      <c r="B51" s="40"/>
-      <c r="C51" s="41"/>
-      <c r="D51" s="41"/>
-      <c r="E51" s="41"/>
-      <c r="F51" s="41"/>
-      <c r="G51" s="41"/>
-      <c r="H51" s="41"/>
-      <c r="I51" s="41"/>
-      <c r="J51" s="41"/>
-      <c r="K51" s="41"/>
-      <c r="L51" s="41"/>
-      <c r="M51" s="41"/>
-      <c r="N51" s="41"/>
-      <c r="O51" s="41"/>
-      <c r="P51" s="41"/>
-      <c r="Q51" s="41"/>
-      <c r="R51" s="41"/>
-      <c r="S51" s="41"/>
-      <c r="T51" s="41"/>
-      <c r="U51" s="41"/>
-      <c r="V51" s="41"/>
-      <c r="W51" s="41"/>
-      <c r="X51" s="41"/>
-      <c r="Y51" s="41"/>
-      <c r="Z51" s="41"/>
-      <c r="AA51" s="42"/>
+      <c r="B51" s="45"/>
+      <c r="C51" s="46"/>
+      <c r="D51" s="46"/>
+      <c r="E51" s="46"/>
+      <c r="F51" s="46"/>
+      <c r="G51" s="46"/>
+      <c r="H51" s="46"/>
+      <c r="I51" s="46"/>
+      <c r="J51" s="46"/>
+      <c r="K51" s="46"/>
+      <c r="L51" s="46"/>
+      <c r="M51" s="46"/>
+      <c r="N51" s="46"/>
+      <c r="O51" s="46"/>
+      <c r="P51" s="46"/>
+      <c r="Q51" s="46"/>
+      <c r="R51" s="46"/>
+      <c r="S51" s="46"/>
+      <c r="T51" s="46"/>
+      <c r="U51" s="46"/>
+      <c r="V51" s="46"/>
+      <c r="W51" s="46"/>
+      <c r="X51" s="46"/>
+      <c r="Y51" s="46"/>
+      <c r="Z51" s="46"/>
+      <c r="AA51" s="47"/>
     </row>
     <row r="52" spans="1:27" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A52" s="30"/>
-      <c r="B52" s="40"/>
-      <c r="C52" s="41"/>
-      <c r="D52" s="41"/>
-      <c r="E52" s="41"/>
-      <c r="F52" s="41"/>
-      <c r="G52" s="41"/>
-      <c r="H52" s="41"/>
-      <c r="I52" s="41"/>
-      <c r="J52" s="41"/>
-      <c r="K52" s="41"/>
-      <c r="L52" s="41"/>
-      <c r="M52" s="41"/>
-      <c r="N52" s="41"/>
-      <c r="O52" s="41"/>
-      <c r="P52" s="41"/>
-      <c r="Q52" s="41"/>
-      <c r="R52" s="41"/>
-      <c r="S52" s="41"/>
-      <c r="T52" s="41"/>
-      <c r="U52" s="41"/>
-      <c r="V52" s="41"/>
-      <c r="W52" s="41"/>
-      <c r="X52" s="41"/>
-      <c r="Y52" s="41"/>
-      <c r="Z52" s="41"/>
-      <c r="AA52" s="42"/>
+      <c r="B52" s="45"/>
+      <c r="C52" s="46"/>
+      <c r="D52" s="46"/>
+      <c r="E52" s="46"/>
+      <c r="F52" s="46"/>
+      <c r="G52" s="46"/>
+      <c r="H52" s="46"/>
+      <c r="I52" s="46"/>
+      <c r="J52" s="46"/>
+      <c r="K52" s="46"/>
+      <c r="L52" s="46"/>
+      <c r="M52" s="46"/>
+      <c r="N52" s="46"/>
+      <c r="O52" s="46"/>
+      <c r="P52" s="46"/>
+      <c r="Q52" s="46"/>
+      <c r="R52" s="46"/>
+      <c r="S52" s="46"/>
+      <c r="T52" s="46"/>
+      <c r="U52" s="46"/>
+      <c r="V52" s="46"/>
+      <c r="W52" s="46"/>
+      <c r="X52" s="46"/>
+      <c r="Y52" s="46"/>
+      <c r="Z52" s="46"/>
+      <c r="AA52" s="47"/>
     </row>
     <row r="53" spans="1:27" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A53" s="30"/>
-      <c r="B53" s="40"/>
-      <c r="C53" s="41"/>
-      <c r="D53" s="41"/>
-      <c r="E53" s="41"/>
-      <c r="F53" s="41"/>
-      <c r="G53" s="41"/>
-      <c r="H53" s="41"/>
-      <c r="I53" s="41"/>
-      <c r="J53" s="41"/>
-      <c r="K53" s="41"/>
-      <c r="L53" s="41"/>
-      <c r="M53" s="41"/>
-      <c r="N53" s="41"/>
-      <c r="O53" s="41"/>
-      <c r="P53" s="41"/>
-      <c r="Q53" s="41"/>
-      <c r="R53" s="41"/>
-      <c r="S53" s="41"/>
-      <c r="T53" s="41"/>
-      <c r="U53" s="41"/>
-      <c r="V53" s="41"/>
-      <c r="W53" s="41"/>
-      <c r="X53" s="41"/>
-      <c r="Y53" s="41"/>
-      <c r="Z53" s="41"/>
-      <c r="AA53" s="42"/>
+      <c r="B53" s="45"/>
+      <c r="C53" s="46"/>
+      <c r="D53" s="46"/>
+      <c r="E53" s="46"/>
+      <c r="F53" s="46"/>
+      <c r="G53" s="46"/>
+      <c r="H53" s="46"/>
+      <c r="I53" s="46"/>
+      <c r="J53" s="46"/>
+      <c r="K53" s="46"/>
+      <c r="L53" s="46"/>
+      <c r="M53" s="46"/>
+      <c r="N53" s="46"/>
+      <c r="O53" s="46"/>
+      <c r="P53" s="46"/>
+      <c r="Q53" s="46"/>
+      <c r="R53" s="46"/>
+      <c r="S53" s="46"/>
+      <c r="T53" s="46"/>
+      <c r="U53" s="46"/>
+      <c r="V53" s="46"/>
+      <c r="W53" s="46"/>
+      <c r="X53" s="46"/>
+      <c r="Y53" s="46"/>
+      <c r="Z53" s="46"/>
+      <c r="AA53" s="47"/>
     </row>
     <row r="54" spans="1:27" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A54" s="30"/>
-      <c r="B54" s="40"/>
-      <c r="C54" s="41"/>
-      <c r="D54" s="41"/>
-      <c r="E54" s="41"/>
-      <c r="F54" s="41"/>
-      <c r="G54" s="41"/>
-      <c r="H54" s="41"/>
-      <c r="I54" s="41"/>
-      <c r="J54" s="41"/>
-      <c r="K54" s="41"/>
-      <c r="L54" s="41"/>
-      <c r="M54" s="41"/>
-      <c r="N54" s="41"/>
-      <c r="O54" s="41"/>
-      <c r="P54" s="41"/>
-      <c r="Q54" s="41"/>
-      <c r="R54" s="41"/>
-      <c r="S54" s="41"/>
-      <c r="T54" s="41"/>
-      <c r="U54" s="41"/>
-      <c r="V54" s="41"/>
-      <c r="W54" s="41"/>
-      <c r="X54" s="41"/>
-      <c r="Y54" s="41"/>
-      <c r="Z54" s="41"/>
-      <c r="AA54" s="42"/>
+      <c r="B54" s="45"/>
+      <c r="C54" s="46"/>
+      <c r="D54" s="46"/>
+      <c r="E54" s="46"/>
+      <c r="F54" s="46"/>
+      <c r="G54" s="46"/>
+      <c r="H54" s="46"/>
+      <c r="I54" s="46"/>
+      <c r="J54" s="46"/>
+      <c r="K54" s="46"/>
+      <c r="L54" s="46"/>
+      <c r="M54" s="46"/>
+      <c r="N54" s="46"/>
+      <c r="O54" s="46"/>
+      <c r="P54" s="46"/>
+      <c r="Q54" s="46"/>
+      <c r="R54" s="46"/>
+      <c r="S54" s="46"/>
+      <c r="T54" s="46"/>
+      <c r="U54" s="46"/>
+      <c r="V54" s="46"/>
+      <c r="W54" s="46"/>
+      <c r="X54" s="46"/>
+      <c r="Y54" s="46"/>
+      <c r="Z54" s="46"/>
+      <c r="AA54" s="47"/>
     </row>
     <row r="55" spans="1:27" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A55" s="30"/>
-      <c r="B55" s="40"/>
-      <c r="C55" s="41"/>
-      <c r="D55" s="41"/>
-      <c r="E55" s="41"/>
-      <c r="F55" s="41"/>
-      <c r="G55" s="41"/>
-      <c r="H55" s="41"/>
-      <c r="I55" s="41"/>
-      <c r="J55" s="41"/>
-      <c r="K55" s="41"/>
-      <c r="L55" s="41"/>
-      <c r="M55" s="41"/>
-      <c r="N55" s="41"/>
-      <c r="O55" s="41"/>
-      <c r="P55" s="41"/>
-      <c r="Q55" s="41"/>
-      <c r="R55" s="41"/>
-      <c r="S55" s="41"/>
-      <c r="T55" s="41"/>
-      <c r="U55" s="41"/>
-      <c r="V55" s="41"/>
-      <c r="W55" s="41"/>
-      <c r="X55" s="41"/>
-      <c r="Y55" s="41"/>
-      <c r="Z55" s="41"/>
-      <c r="AA55" s="42"/>
+      <c r="B55" s="45"/>
+      <c r="C55" s="46"/>
+      <c r="D55" s="46"/>
+      <c r="E55" s="46"/>
+      <c r="F55" s="46"/>
+      <c r="G55" s="46"/>
+      <c r="H55" s="46"/>
+      <c r="I55" s="46"/>
+      <c r="J55" s="46"/>
+      <c r="K55" s="46"/>
+      <c r="L55" s="46"/>
+      <c r="M55" s="46"/>
+      <c r="N55" s="46"/>
+      <c r="O55" s="46"/>
+      <c r="P55" s="46"/>
+      <c r="Q55" s="46"/>
+      <c r="R55" s="46"/>
+      <c r="S55" s="46"/>
+      <c r="T55" s="46"/>
+      <c r="U55" s="46"/>
+      <c r="V55" s="46"/>
+      <c r="W55" s="46"/>
+      <c r="X55" s="46"/>
+      <c r="Y55" s="46"/>
+      <c r="Z55" s="46"/>
+      <c r="AA55" s="47"/>
     </row>
     <row r="56" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A56" s="1"/>
@@ -3000,15 +2999,15 @@
     </row>
     <row r="58" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A58" s="1"/>
-      <c r="B58" s="72"/>
-      <c r="C58" s="72"/>
-      <c r="D58" s="72"/>
-      <c r="E58" s="72"/>
-      <c r="F58" s="72"/>
-      <c r="G58" s="72"/>
-      <c r="H58" s="72"/>
-      <c r="I58" s="72"/>
-      <c r="J58" s="72"/>
+      <c r="B58" s="1"/>
+      <c r="C58" s="1"/>
+      <c r="D58" s="1"/>
+      <c r="E58" s="1"/>
+      <c r="F58" s="1"/>
+      <c r="G58" s="1"/>
+      <c r="H58" s="1"/>
+      <c r="I58" s="1"/>
+      <c r="J58" s="1"/>
       <c r="K58" s="36"/>
       <c r="L58" s="36"/>
       <c r="M58" s="36"/>
@@ -3029,25 +3028,25 @@
     </row>
     <row r="59" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A59" s="1"/>
-      <c r="B59" s="72"/>
-      <c r="C59" s="72"/>
-      <c r="D59" s="72"/>
-      <c r="E59" s="72"/>
-      <c r="F59" s="72"/>
-      <c r="G59" s="72"/>
-      <c r="H59" s="72"/>
-      <c r="I59" s="72"/>
-      <c r="J59" s="72"/>
-      <c r="K59" s="67"/>
-      <c r="L59" s="68"/>
-      <c r="M59" s="68"/>
-      <c r="N59" s="68"/>
-      <c r="O59" s="68"/>
-      <c r="P59" s="68"/>
-      <c r="Q59" s="68"/>
-      <c r="R59" s="35"/>
-      <c r="S59" s="35"/>
-      <c r="T59" s="35"/>
+      <c r="B59" s="1"/>
+      <c r="C59" s="1"/>
+      <c r="D59" s="1"/>
+      <c r="E59" s="51"/>
+      <c r="F59" s="51"/>
+      <c r="G59" s="51"/>
+      <c r="H59" s="51"/>
+      <c r="I59" s="51"/>
+      <c r="J59" s="51"/>
+      <c r="K59" s="51"/>
+      <c r="L59" s="51"/>
+      <c r="M59" s="51"/>
+      <c r="N59" s="51"/>
+      <c r="O59" s="51"/>
+      <c r="P59" s="51"/>
+      <c r="Q59" s="71"/>
+      <c r="R59" s="71"/>
+      <c r="S59" s="71"/>
+      <c r="T59" s="71"/>
       <c r="U59" s="35"/>
       <c r="V59" s="35"/>
       <c r="W59" s="35"/>
@@ -3205,61 +3204,61 @@
     <row r="65" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A65" s="1"/>
       <c r="B65" s="34"/>
-      <c r="C65" s="66" t="s">
+      <c r="C65" s="40" t="s">
         <v>14</v>
       </c>
-      <c r="D65" s="56"/>
-      <c r="E65" s="56"/>
-      <c r="F65" s="56"/>
-      <c r="G65" s="56"/>
-      <c r="H65" s="56"/>
-      <c r="I65" s="56"/>
-      <c r="J65" s="56"/>
-      <c r="K65" s="56"/>
-      <c r="L65" s="56"/>
-      <c r="M65" s="56"/>
-      <c r="N65" s="56"/>
-      <c r="O65" s="56"/>
-      <c r="P65" s="56"/>
-      <c r="Q65" s="56"/>
-      <c r="R65" s="56"/>
-      <c r="S65" s="56"/>
-      <c r="T65" s="56"/>
-      <c r="U65" s="56"/>
-      <c r="V65" s="56"/>
-      <c r="W65" s="56"/>
-      <c r="X65" s="56"/>
-      <c r="Y65" s="56"/>
-      <c r="Z65" s="56"/>
+      <c r="D65" s="41"/>
+      <c r="E65" s="41"/>
+      <c r="F65" s="41"/>
+      <c r="G65" s="41"/>
+      <c r="H65" s="41"/>
+      <c r="I65" s="41"/>
+      <c r="J65" s="41"/>
+      <c r="K65" s="41"/>
+      <c r="L65" s="41"/>
+      <c r="M65" s="41"/>
+      <c r="N65" s="41"/>
+      <c r="O65" s="41"/>
+      <c r="P65" s="41"/>
+      <c r="Q65" s="41"/>
+      <c r="R65" s="41"/>
+      <c r="S65" s="41"/>
+      <c r="T65" s="41"/>
+      <c r="U65" s="41"/>
+      <c r="V65" s="41"/>
+      <c r="W65" s="41"/>
+      <c r="X65" s="41"/>
+      <c r="Y65" s="41"/>
+      <c r="Z65" s="41"/>
       <c r="AA65" s="34"/>
     </row>
     <row r="66" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A66" s="1"/>
       <c r="B66" s="34"/>
-      <c r="C66" s="56"/>
-      <c r="D66" s="56"/>
-      <c r="E66" s="56"/>
-      <c r="F66" s="56"/>
-      <c r="G66" s="56"/>
-      <c r="H66" s="56"/>
-      <c r="I66" s="56"/>
-      <c r="J66" s="56"/>
-      <c r="K66" s="56"/>
-      <c r="L66" s="56"/>
-      <c r="M66" s="56"/>
-      <c r="N66" s="56"/>
-      <c r="O66" s="56"/>
-      <c r="P66" s="56"/>
-      <c r="Q66" s="56"/>
-      <c r="R66" s="56"/>
-      <c r="S66" s="56"/>
-      <c r="T66" s="56"/>
-      <c r="U66" s="56"/>
-      <c r="V66" s="56"/>
-      <c r="W66" s="56"/>
-      <c r="X66" s="56"/>
-      <c r="Y66" s="56"/>
-      <c r="Z66" s="56"/>
+      <c r="C66" s="41"/>
+      <c r="D66" s="41"/>
+      <c r="E66" s="41"/>
+      <c r="F66" s="41"/>
+      <c r="G66" s="41"/>
+      <c r="H66" s="41"/>
+      <c r="I66" s="41"/>
+      <c r="J66" s="41"/>
+      <c r="K66" s="41"/>
+      <c r="L66" s="41"/>
+      <c r="M66" s="41"/>
+      <c r="N66" s="41"/>
+      <c r="O66" s="41"/>
+      <c r="P66" s="41"/>
+      <c r="Q66" s="41"/>
+      <c r="R66" s="41"/>
+      <c r="S66" s="41"/>
+      <c r="T66" s="41"/>
+      <c r="U66" s="41"/>
+      <c r="V66" s="41"/>
+      <c r="W66" s="41"/>
+      <c r="X66" s="41"/>
+      <c r="Y66" s="41"/>
+      <c r="Z66" s="41"/>
       <c r="AA66" s="34"/>
     </row>
     <row r="67" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -30350,30 +30349,15 @@
     </row>
   </sheetData>
   <mergeCells count="50">
-    <mergeCell ref="C65:Z66"/>
-    <mergeCell ref="B40:AA40"/>
-    <mergeCell ref="B49:AA49"/>
-    <mergeCell ref="K59:Q59"/>
-    <mergeCell ref="B55:AA55"/>
-    <mergeCell ref="B42:AA42"/>
-    <mergeCell ref="B54:AA54"/>
-    <mergeCell ref="B48:AA48"/>
-    <mergeCell ref="B58:J59"/>
-    <mergeCell ref="H10:Z10"/>
-    <mergeCell ref="B51:AA51"/>
-    <mergeCell ref="B44:AA44"/>
-    <mergeCell ref="B53:AA53"/>
-    <mergeCell ref="B38:AA38"/>
-    <mergeCell ref="B29:AA29"/>
-    <mergeCell ref="H21:Z21"/>
-    <mergeCell ref="B34:AA34"/>
-    <mergeCell ref="B37:AA37"/>
-    <mergeCell ref="B28:AA28"/>
-    <mergeCell ref="B24:AA24"/>
-    <mergeCell ref="B30:AA30"/>
-    <mergeCell ref="H17:Z17"/>
-    <mergeCell ref="B47:AA47"/>
-    <mergeCell ref="B52:AA52"/>
+    <mergeCell ref="B32:AA32"/>
+    <mergeCell ref="B50:AA50"/>
+    <mergeCell ref="B14:AA15"/>
+    <mergeCell ref="B26:AA26"/>
+    <mergeCell ref="B41:AA41"/>
+    <mergeCell ref="H19:Z19"/>
+    <mergeCell ref="B33:AA33"/>
+    <mergeCell ref="B17:G17"/>
+    <mergeCell ref="B23:AA23"/>
     <mergeCell ref="B3:AA3"/>
     <mergeCell ref="B19:G19"/>
     <mergeCell ref="B31:AA31"/>
@@ -30390,16 +30374,31 @@
     <mergeCell ref="H12:T12"/>
     <mergeCell ref="B25:AA25"/>
     <mergeCell ref="B45:AA45"/>
+    <mergeCell ref="H10:Z10"/>
+    <mergeCell ref="B51:AA51"/>
+    <mergeCell ref="B44:AA44"/>
+    <mergeCell ref="B53:AA53"/>
+    <mergeCell ref="B38:AA38"/>
+    <mergeCell ref="B29:AA29"/>
+    <mergeCell ref="H21:Z21"/>
+    <mergeCell ref="B34:AA34"/>
+    <mergeCell ref="B37:AA37"/>
+    <mergeCell ref="B28:AA28"/>
+    <mergeCell ref="B24:AA24"/>
+    <mergeCell ref="B30:AA30"/>
+    <mergeCell ref="H17:Z17"/>
+    <mergeCell ref="B47:AA47"/>
+    <mergeCell ref="B52:AA52"/>
     <mergeCell ref="B36:AA36"/>
-    <mergeCell ref="B32:AA32"/>
-    <mergeCell ref="B50:AA50"/>
-    <mergeCell ref="B14:AA15"/>
-    <mergeCell ref="B26:AA26"/>
-    <mergeCell ref="B41:AA41"/>
-    <mergeCell ref="H19:Z19"/>
-    <mergeCell ref="B33:AA33"/>
-    <mergeCell ref="B17:G17"/>
-    <mergeCell ref="B23:AA23"/>
+    <mergeCell ref="C65:Z66"/>
+    <mergeCell ref="B40:AA40"/>
+    <mergeCell ref="B49:AA49"/>
+    <mergeCell ref="B55:AA55"/>
+    <mergeCell ref="B42:AA42"/>
+    <mergeCell ref="B54:AA54"/>
+    <mergeCell ref="B48:AA48"/>
+    <mergeCell ref="E59:P59"/>
+    <mergeCell ref="Q59:T59"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.39370078740157483" bottom="0.98425196850393704" header="0" footer="0"/>

</xml_diff>